<commit_message>
Updates to 3/10 smelt assessment
</commit_message>
<xml_diff>
--- a/data_raw/smelt/SLS catch update 3.10.26.xlsx
+++ b/data_raw/smelt/SLS catch update 3.10.26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lmccormick_usbr_gov/Documents/Documents/Research/R/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{AC0A6D38-CDE9-4EFA-A007-215466C74972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B95AE1F-FC8B-4910-8781-8D39AC4B47BF}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{AC0A6D38-CDE9-4EFA-A007-215466C74972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1712969B-5F54-4754-84EE-6FB9B64847AA}"/>
   <bookViews>
     <workbookView xWindow="-18336" yWindow="-15840" windowWidth="21672" windowHeight="11676" activeTab="6" xr2:uid="{E318DA66-929E-4160-AE8F-A3EAE62CC340}"/>
   </bookViews>
@@ -2017,6 +2017,9 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="1" fillId="5" borderId="3" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="24" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -2052,9 +2055,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="5" borderId="3" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2618,7 +2618,7 @@
       <c r="M3" s="42"/>
       <c r="N3" s="43"/>
       <c r="O3" s="44"/>
-      <c r="P3" s="343" t="s">
+      <c r="P3" s="344" t="s">
         <v>31</v>
       </c>
       <c r="Q3" s="13"/>
@@ -2659,7 +2659,7 @@
       <c r="M4" s="52"/>
       <c r="N4" s="53"/>
       <c r="O4" s="54"/>
-      <c r="P4" s="343"/>
+      <c r="P4" s="344"/>
       <c r="Q4" s="13"/>
     </row>
     <row r="5" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2698,7 +2698,7 @@
       <c r="M5" s="59"/>
       <c r="N5" s="60"/>
       <c r="O5" s="61"/>
-      <c r="P5" s="343"/>
+      <c r="P5" s="344"/>
       <c r="Q5" s="13"/>
     </row>
     <row r="6" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2737,7 +2737,7 @@
       <c r="M6" s="59"/>
       <c r="N6" s="60"/>
       <c r="O6" s="61"/>
-      <c r="P6" s="343"/>
+      <c r="P6" s="344"/>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2776,7 +2776,7 @@
       <c r="M7" s="59"/>
       <c r="N7" s="60"/>
       <c r="O7" s="61"/>
-      <c r="P7" s="343"/>
+      <c r="P7" s="344"/>
       <c r="Q7" s="13"/>
     </row>
     <row r="8" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2815,7 +2815,7 @@
       <c r="M8" s="59"/>
       <c r="N8" s="60"/>
       <c r="O8" s="61"/>
-      <c r="P8" s="343"/>
+      <c r="P8" s="344"/>
       <c r="Q8" s="13"/>
     </row>
     <row r="9" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2854,7 +2854,7 @@
       <c r="M9" s="59"/>
       <c r="N9" s="60"/>
       <c r="O9" s="61"/>
-      <c r="P9" s="343"/>
+      <c r="P9" s="344"/>
       <c r="Q9" s="13"/>
     </row>
     <row r="10" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2893,7 +2893,7 @@
       <c r="M10" s="59"/>
       <c r="N10" s="60"/>
       <c r="O10" s="61"/>
-      <c r="P10" s="343"/>
+      <c r="P10" s="344"/>
       <c r="Q10" s="13"/>
     </row>
     <row r="11" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2932,7 +2932,7 @@
       <c r="M11" s="59"/>
       <c r="N11" s="60"/>
       <c r="O11" s="61"/>
-      <c r="P11" s="343"/>
+      <c r="P11" s="344"/>
       <c r="Q11" s="13"/>
     </row>
     <row r="12" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2971,7 +2971,7 @@
       <c r="M12" s="59"/>
       <c r="N12" s="60"/>
       <c r="O12" s="61"/>
-      <c r="P12" s="343"/>
+      <c r="P12" s="344"/>
       <c r="Q12" s="13"/>
     </row>
     <row r="13" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3010,7 +3010,7 @@
       <c r="M13" s="59"/>
       <c r="N13" s="60"/>
       <c r="O13" s="61"/>
-      <c r="P13" s="343"/>
+      <c r="P13" s="344"/>
       <c r="Q13" s="13"/>
     </row>
     <row r="14" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3049,7 +3049,7 @@
       <c r="M14" s="59"/>
       <c r="N14" s="60"/>
       <c r="O14" s="61"/>
-      <c r="P14" s="343"/>
+      <c r="P14" s="344"/>
       <c r="Q14" s="13"/>
     </row>
     <row r="15" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3088,7 +3088,7 @@
       <c r="M15" s="66"/>
       <c r="N15" s="67"/>
       <c r="O15" s="68"/>
-      <c r="P15" s="343"/>
+      <c r="P15" s="344"/>
       <c r="Q15" s="13"/>
     </row>
     <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3127,7 +3127,7 @@
       <c r="M16" s="74"/>
       <c r="N16" s="75"/>
       <c r="O16" s="76"/>
-      <c r="P16" s="344" t="s">
+      <c r="P16" s="345" t="s">
         <v>12</v>
       </c>
       <c r="Q16" s="13"/>
@@ -3168,7 +3168,7 @@
       <c r="M17" s="82"/>
       <c r="N17" s="83"/>
       <c r="O17" s="84"/>
-      <c r="P17" s="345"/>
+      <c r="P17" s="346"/>
       <c r="Q17" s="13"/>
     </row>
     <row r="18" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3207,7 +3207,7 @@
       <c r="M18" s="82"/>
       <c r="N18" s="83"/>
       <c r="O18" s="84"/>
-      <c r="P18" s="345"/>
+      <c r="P18" s="346"/>
       <c r="Q18" s="13"/>
     </row>
     <row r="19" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3246,7 +3246,7 @@
       <c r="M19" s="82"/>
       <c r="N19" s="83"/>
       <c r="O19" s="84"/>
-      <c r="P19" s="345"/>
+      <c r="P19" s="346"/>
       <c r="Q19" s="13"/>
     </row>
     <row r="20" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3285,7 +3285,7 @@
       <c r="M20" s="82"/>
       <c r="N20" s="83"/>
       <c r="O20" s="84"/>
-      <c r="P20" s="345"/>
+      <c r="P20" s="346"/>
       <c r="Q20" s="13"/>
     </row>
     <row r="21" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3324,7 +3324,7 @@
       <c r="M21" s="82"/>
       <c r="N21" s="83"/>
       <c r="O21" s="84"/>
-      <c r="P21" s="345"/>
+      <c r="P21" s="346"/>
       <c r="Q21" s="13"/>
     </row>
     <row r="22" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3363,7 +3363,7 @@
       <c r="M22" s="82"/>
       <c r="N22" s="83"/>
       <c r="O22" s="84"/>
-      <c r="P22" s="345"/>
+      <c r="P22" s="346"/>
       <c r="Q22" s="13"/>
     </row>
     <row r="23" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3402,7 +3402,7 @@
       <c r="M23" s="82"/>
       <c r="N23" s="91"/>
       <c r="O23" s="92"/>
-      <c r="P23" s="345"/>
+      <c r="P23" s="346"/>
       <c r="Q23" s="13"/>
     </row>
     <row r="24" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3441,7 +3441,7 @@
       <c r="M24" s="98"/>
       <c r="N24" s="99"/>
       <c r="O24" s="100"/>
-      <c r="P24" s="346"/>
+      <c r="P24" s="347"/>
       <c r="Q24" s="13"/>
     </row>
     <row r="25" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3480,7 +3480,7 @@
       <c r="M25" s="106"/>
       <c r="N25" s="107"/>
       <c r="O25" s="108"/>
-      <c r="P25" s="347" t="s">
+      <c r="P25" s="348" t="s">
         <v>32</v>
       </c>
       <c r="Q25" s="13"/>
@@ -3521,7 +3521,7 @@
       <c r="M26" s="113"/>
       <c r="N26" s="114"/>
       <c r="O26" s="115"/>
-      <c r="P26" s="347"/>
+      <c r="P26" s="348"/>
       <c r="Q26" s="13"/>
     </row>
     <row r="27" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3560,7 +3560,7 @@
       <c r="M27" s="120"/>
       <c r="N27" s="121"/>
       <c r="O27" s="122"/>
-      <c r="P27" s="347"/>
+      <c r="P27" s="348"/>
       <c r="Q27" s="13"/>
     </row>
     <row r="28" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3599,7 +3599,7 @@
       <c r="M28" s="127"/>
       <c r="N28" s="128"/>
       <c r="O28" s="129"/>
-      <c r="P28" s="348" t="s">
+      <c r="P28" s="349" t="s">
         <v>33</v>
       </c>
       <c r="Q28" s="13"/>
@@ -3640,7 +3640,7 @@
       <c r="M29" s="134"/>
       <c r="N29" s="135"/>
       <c r="O29" s="136"/>
-      <c r="P29" s="348"/>
+      <c r="P29" s="349"/>
       <c r="Q29" s="13"/>
     </row>
     <row r="30" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3679,7 +3679,7 @@
       <c r="M30" s="134"/>
       <c r="N30" s="135"/>
       <c r="O30" s="136"/>
-      <c r="P30" s="348"/>
+      <c r="P30" s="349"/>
       <c r="Q30" s="13"/>
     </row>
     <row r="31" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3718,7 +3718,7 @@
       <c r="M31" s="134"/>
       <c r="N31" s="135"/>
       <c r="O31" s="136"/>
-      <c r="P31" s="348"/>
+      <c r="P31" s="349"/>
       <c r="Q31" s="13"/>
     </row>
     <row r="32" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3757,7 +3757,7 @@
       <c r="M32" s="134"/>
       <c r="N32" s="135"/>
       <c r="O32" s="136"/>
-      <c r="P32" s="348"/>
+      <c r="P32" s="349"/>
       <c r="Q32" s="13"/>
     </row>
     <row r="33" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3796,7 +3796,7 @@
       <c r="M33" s="134"/>
       <c r="N33" s="135"/>
       <c r="O33" s="136"/>
-      <c r="P33" s="348"/>
+      <c r="P33" s="349"/>
       <c r="Q33" s="13"/>
     </row>
     <row r="34" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3835,7 +3835,7 @@
       <c r="M34" s="134"/>
       <c r="N34" s="135"/>
       <c r="O34" s="136"/>
-      <c r="P34" s="348"/>
+      <c r="P34" s="349"/>
       <c r="Q34" s="13"/>
     </row>
     <row r="35" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3874,7 +3874,7 @@
       <c r="M35" s="134"/>
       <c r="N35" s="135"/>
       <c r="O35" s="136"/>
-      <c r="P35" s="348"/>
+      <c r="P35" s="349"/>
       <c r="Q35" s="13"/>
     </row>
     <row r="36" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3913,7 +3913,7 @@
       <c r="M36" s="145"/>
       <c r="N36" s="146"/>
       <c r="O36" s="147"/>
-      <c r="P36" s="348"/>
+      <c r="P36" s="349"/>
       <c r="Q36" s="13"/>
     </row>
     <row r="37" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3952,7 +3952,7 @@
       <c r="M37" s="154"/>
       <c r="N37" s="155"/>
       <c r="O37" s="156"/>
-      <c r="P37" s="349" t="s">
+      <c r="P37" s="350" t="s">
         <v>13</v>
       </c>
       <c r="Q37" s="13"/>
@@ -3993,7 +3993,7 @@
       <c r="M38" s="162"/>
       <c r="N38" s="163"/>
       <c r="O38" s="164"/>
-      <c r="P38" s="349"/>
+      <c r="P38" s="350"/>
       <c r="Q38" s="13"/>
     </row>
     <row r="39" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4032,7 +4032,7 @@
       <c r="M39" s="162"/>
       <c r="N39" s="163"/>
       <c r="O39" s="164"/>
-      <c r="P39" s="349"/>
+      <c r="P39" s="350"/>
       <c r="Q39" s="13"/>
     </row>
     <row r="40" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4071,7 +4071,7 @@
       <c r="M40" s="162"/>
       <c r="N40" s="163"/>
       <c r="O40" s="164"/>
-      <c r="P40" s="349"/>
+      <c r="P40" s="350"/>
       <c r="Q40" s="13"/>
     </row>
     <row r="41" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4110,7 +4110,7 @@
       <c r="M41" s="171"/>
       <c r="N41" s="172"/>
       <c r="O41" s="173"/>
-      <c r="P41" s="349"/>
+      <c r="P41" s="350"/>
       <c r="Q41" s="13"/>
     </row>
     <row r="42" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -4149,7 +4149,7 @@
       <c r="M42" s="181"/>
       <c r="N42" s="182"/>
       <c r="O42" s="183"/>
-      <c r="P42" s="350" t="s">
+      <c r="P42" s="351" t="s">
         <v>34</v>
       </c>
       <c r="Q42" s="13"/>
@@ -4190,7 +4190,7 @@
       <c r="M43" s="190"/>
       <c r="N43" s="191"/>
       <c r="O43" s="192"/>
-      <c r="P43" s="351"/>
+      <c r="P43" s="352"/>
       <c r="Q43" s="13"/>
     </row>
     <row r="44" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -4229,7 +4229,7 @@
       <c r="M44" s="190"/>
       <c r="N44" s="191"/>
       <c r="O44" s="192"/>
-      <c r="P44" s="351"/>
+      <c r="P44" s="352"/>
       <c r="Q44" s="13"/>
     </row>
     <row r="45" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -4268,7 +4268,7 @@
       <c r="M45" s="190"/>
       <c r="N45" s="191"/>
       <c r="O45" s="192"/>
-      <c r="P45" s="351"/>
+      <c r="P45" s="352"/>
       <c r="Q45" s="13"/>
     </row>
     <row r="46" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -4307,7 +4307,7 @@
       <c r="M46" s="190"/>
       <c r="N46" s="191"/>
       <c r="O46" s="192"/>
-      <c r="P46" s="351"/>
+      <c r="P46" s="352"/>
       <c r="Q46" s="13"/>
     </row>
     <row r="47" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -4346,7 +4346,7 @@
       <c r="M47" s="190"/>
       <c r="N47" s="191"/>
       <c r="O47" s="192"/>
-      <c r="P47" s="351"/>
+      <c r="P47" s="352"/>
       <c r="Q47" s="13"/>
     </row>
     <row r="48" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -4385,7 +4385,7 @@
       <c r="M48" s="198"/>
       <c r="N48" s="199"/>
       <c r="O48" s="200"/>
-      <c r="P48" s="351"/>
+      <c r="P48" s="352"/>
       <c r="Q48" s="13"/>
     </row>
     <row r="49" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4424,7 +4424,7 @@
       <c r="M49" s="201"/>
       <c r="N49" s="202"/>
       <c r="O49" s="203"/>
-      <c r="P49" s="352"/>
+      <c r="P49" s="353"/>
       <c r="Q49" s="13"/>
     </row>
     <row r="50" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4462,7 +4462,7 @@
       <c r="M50" s="210"/>
       <c r="N50" s="211"/>
       <c r="O50" s="212"/>
-      <c r="P50" s="342" t="s">
+      <c r="P50" s="343" t="s">
         <v>28</v>
       </c>
       <c r="Q50" s="13"/>
@@ -4503,7 +4503,7 @@
       <c r="M51" s="219"/>
       <c r="N51" s="220"/>
       <c r="O51" s="221"/>
-      <c r="P51" s="342"/>
+      <c r="P51" s="343"/>
       <c r="Q51" s="13"/>
     </row>
     <row r="52" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4542,7 +4542,7 @@
       <c r="M52" s="229"/>
       <c r="N52" s="230"/>
       <c r="O52" s="231"/>
-      <c r="P52" s="342"/>
+      <c r="P52" s="343"/>
       <c r="Q52" s="13"/>
     </row>
     <row r="53" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4581,7 +4581,7 @@
       <c r="M53" s="229"/>
       <c r="N53" s="230"/>
       <c r="O53" s="231"/>
-      <c r="P53" s="342"/>
+      <c r="P53" s="343"/>
       <c r="Q53" s="13"/>
     </row>
     <row r="54" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4620,7 +4620,7 @@
       <c r="M54" s="229"/>
       <c r="N54" s="230"/>
       <c r="O54" s="231"/>
-      <c r="P54" s="342"/>
+      <c r="P54" s="343"/>
       <c r="Q54" s="13"/>
     </row>
     <row r="55" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4657,7 +4657,7 @@
       <c r="M55" s="229"/>
       <c r="N55" s="230"/>
       <c r="O55" s="231"/>
-      <c r="P55" s="342"/>
+      <c r="P55" s="343"/>
       <c r="Q55" s="13"/>
     </row>
     <row r="56" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4696,7 +4696,7 @@
       <c r="M56" s="229"/>
       <c r="N56" s="230"/>
       <c r="O56" s="231"/>
-      <c r="P56" s="342"/>
+      <c r="P56" s="343"/>
       <c r="Q56" s="13"/>
     </row>
     <row r="57" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4735,7 +4735,7 @@
       <c r="M57" s="229"/>
       <c r="N57" s="230"/>
       <c r="O57" s="231"/>
-      <c r="P57" s="342"/>
+      <c r="P57" s="343"/>
       <c r="Q57" s="13"/>
     </row>
     <row r="58" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4772,7 +4772,7 @@
       <c r="M58" s="229"/>
       <c r="N58" s="230"/>
       <c r="O58" s="231"/>
-      <c r="P58" s="342"/>
+      <c r="P58" s="343"/>
       <c r="Q58" s="13"/>
     </row>
     <row r="59" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4809,7 +4809,7 @@
       <c r="M59" s="229"/>
       <c r="N59" s="230"/>
       <c r="O59" s="231"/>
-      <c r="P59" s="342"/>
+      <c r="P59" s="343"/>
       <c r="Q59" s="13"/>
     </row>
     <row r="60" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4848,7 +4848,7 @@
       <c r="M60" s="229"/>
       <c r="N60" s="230"/>
       <c r="O60" s="231"/>
-      <c r="P60" s="342"/>
+      <c r="P60" s="343"/>
       <c r="Q60" s="13"/>
     </row>
     <row r="61" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4885,7 +4885,7 @@
       <c r="M61" s="239"/>
       <c r="N61" s="240"/>
       <c r="O61" s="241"/>
-      <c r="P61" s="342"/>
+      <c r="P61" s="343"/>
       <c r="Q61" s="13"/>
     </row>
     <row r="62" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -5360,7 +5360,7 @@
       <c r="M3" s="242"/>
       <c r="N3" s="43"/>
       <c r="O3" s="267"/>
-      <c r="P3" s="343" t="s">
+      <c r="P3" s="344" t="s">
         <v>31</v>
       </c>
       <c r="Q3" s="13"/>
@@ -5401,7 +5401,7 @@
       <c r="M4" s="243"/>
       <c r="N4" s="53"/>
       <c r="O4" s="268"/>
-      <c r="P4" s="343"/>
+      <c r="P4" s="344"/>
       <c r="Q4" s="13"/>
     </row>
     <row r="5" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -5440,7 +5440,7 @@
       <c r="M5" s="244"/>
       <c r="N5" s="60"/>
       <c r="O5" s="269"/>
-      <c r="P5" s="343"/>
+      <c r="P5" s="344"/>
       <c r="Q5" s="13"/>
     </row>
     <row r="6" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -5479,7 +5479,7 @@
       <c r="M6" s="244"/>
       <c r="N6" s="60"/>
       <c r="O6" s="269"/>
-      <c r="P6" s="343"/>
+      <c r="P6" s="344"/>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -5518,7 +5518,7 @@
       <c r="M7" s="244"/>
       <c r="N7" s="60"/>
       <c r="O7" s="269"/>
-      <c r="P7" s="343"/>
+      <c r="P7" s="344"/>
       <c r="Q7" s="13"/>
     </row>
     <row r="8" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -5557,7 +5557,7 @@
       <c r="M8" s="244"/>
       <c r="N8" s="60"/>
       <c r="O8" s="269"/>
-      <c r="P8" s="343"/>
+      <c r="P8" s="344"/>
       <c r="Q8" s="13"/>
     </row>
     <row r="9" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -5596,7 +5596,7 @@
       <c r="M9" s="244"/>
       <c r="N9" s="60"/>
       <c r="O9" s="269"/>
-      <c r="P9" s="343"/>
+      <c r="P9" s="344"/>
       <c r="Q9" s="13"/>
     </row>
     <row r="10" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -5635,7 +5635,7 @@
       <c r="M10" s="244"/>
       <c r="N10" s="60"/>
       <c r="O10" s="269"/>
-      <c r="P10" s="343"/>
+      <c r="P10" s="344"/>
       <c r="Q10" s="13"/>
     </row>
     <row r="11" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -5674,7 +5674,7 @@
       <c r="M11" s="244"/>
       <c r="N11" s="60"/>
       <c r="O11" s="269"/>
-      <c r="P11" s="343"/>
+      <c r="P11" s="344"/>
       <c r="Q11" s="13"/>
     </row>
     <row r="12" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -5713,7 +5713,7 @@
       <c r="M12" s="244"/>
       <c r="N12" s="60"/>
       <c r="O12" s="269"/>
-      <c r="P12" s="343"/>
+      <c r="P12" s="344"/>
       <c r="Q12" s="13"/>
     </row>
     <row r="13" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -5752,7 +5752,7 @@
       <c r="M13" s="244"/>
       <c r="N13" s="60"/>
       <c r="O13" s="269"/>
-      <c r="P13" s="343"/>
+      <c r="P13" s="344"/>
       <c r="Q13" s="13"/>
     </row>
     <row r="14" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -5791,7 +5791,7 @@
       <c r="M14" s="244"/>
       <c r="N14" s="60"/>
       <c r="O14" s="269"/>
-      <c r="P14" s="343"/>
+      <c r="P14" s="344"/>
       <c r="Q14" s="13"/>
     </row>
     <row r="15" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -5830,7 +5830,7 @@
       <c r="M15" s="245"/>
       <c r="N15" s="67"/>
       <c r="O15" s="270"/>
-      <c r="P15" s="343"/>
+      <c r="P15" s="344"/>
       <c r="Q15" s="13"/>
     </row>
     <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -5869,7 +5869,7 @@
       <c r="M16" s="246"/>
       <c r="N16" s="75"/>
       <c r="O16" s="271"/>
-      <c r="P16" s="344" t="s">
+      <c r="P16" s="345" t="s">
         <v>12</v>
       </c>
       <c r="Q16" s="13"/>
@@ -5910,7 +5910,7 @@
       <c r="M17" s="247"/>
       <c r="N17" s="83"/>
       <c r="O17" s="272"/>
-      <c r="P17" s="345"/>
+      <c r="P17" s="346"/>
       <c r="Q17" s="13"/>
     </row>
     <row r="18" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -5949,7 +5949,7 @@
       <c r="M18" s="247"/>
       <c r="N18" s="83"/>
       <c r="O18" s="272"/>
-      <c r="P18" s="345"/>
+      <c r="P18" s="346"/>
       <c r="Q18" s="13"/>
     </row>
     <row r="19" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -5988,7 +5988,7 @@
       <c r="M19" s="247"/>
       <c r="N19" s="83"/>
       <c r="O19" s="272"/>
-      <c r="P19" s="345"/>
+      <c r="P19" s="346"/>
       <c r="Q19" s="13"/>
     </row>
     <row r="20" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -6027,7 +6027,7 @@
       <c r="M20" s="247"/>
       <c r="N20" s="83"/>
       <c r="O20" s="272"/>
-      <c r="P20" s="345"/>
+      <c r="P20" s="346"/>
       <c r="Q20" s="13"/>
     </row>
     <row r="21" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -6066,7 +6066,7 @@
       <c r="M21" s="247"/>
       <c r="N21" s="83"/>
       <c r="O21" s="272"/>
-      <c r="P21" s="345"/>
+      <c r="P21" s="346"/>
       <c r="Q21" s="13"/>
     </row>
     <row r="22" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -6105,7 +6105,7 @@
       <c r="M22" s="247"/>
       <c r="N22" s="83"/>
       <c r="O22" s="272"/>
-      <c r="P22" s="345"/>
+      <c r="P22" s="346"/>
       <c r="Q22" s="13"/>
     </row>
     <row r="23" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -6144,7 +6144,7 @@
       <c r="M23" s="247"/>
       <c r="N23" s="91"/>
       <c r="O23" s="273"/>
-      <c r="P23" s="345"/>
+      <c r="P23" s="346"/>
       <c r="Q23" s="13"/>
     </row>
     <row r="24" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6183,7 +6183,7 @@
       <c r="M24" s="248"/>
       <c r="N24" s="99"/>
       <c r="O24" s="274"/>
-      <c r="P24" s="346"/>
+      <c r="P24" s="347"/>
       <c r="Q24" s="13"/>
     </row>
     <row r="25" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6222,7 +6222,7 @@
       <c r="M25" s="249"/>
       <c r="N25" s="107"/>
       <c r="O25" s="275"/>
-      <c r="P25" s="347" t="s">
+      <c r="P25" s="348" t="s">
         <v>32</v>
       </c>
       <c r="Q25" s="13"/>
@@ -6263,7 +6263,7 @@
       <c r="M26" s="250"/>
       <c r="N26" s="114"/>
       <c r="O26" s="276"/>
-      <c r="P26" s="347"/>
+      <c r="P26" s="348"/>
       <c r="Q26" s="13"/>
     </row>
     <row r="27" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6302,7 +6302,7 @@
       <c r="M27" s="251"/>
       <c r="N27" s="121"/>
       <c r="O27" s="277"/>
-      <c r="P27" s="347"/>
+      <c r="P27" s="348"/>
       <c r="Q27" s="13"/>
     </row>
     <row r="28" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6341,7 +6341,7 @@
       <c r="M28" s="252"/>
       <c r="N28" s="128"/>
       <c r="O28" s="278"/>
-      <c r="P28" s="348" t="s">
+      <c r="P28" s="349" t="s">
         <v>33</v>
       </c>
       <c r="Q28" s="13"/>
@@ -6382,7 +6382,7 @@
       <c r="M29" s="253"/>
       <c r="N29" s="135"/>
       <c r="O29" s="279"/>
-      <c r="P29" s="348"/>
+      <c r="P29" s="349"/>
       <c r="Q29" s="13"/>
     </row>
     <row r="30" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6421,7 +6421,7 @@
       <c r="M30" s="253"/>
       <c r="N30" s="135"/>
       <c r="O30" s="279"/>
-      <c r="P30" s="348"/>
+      <c r="P30" s="349"/>
       <c r="Q30" s="13"/>
     </row>
     <row r="31" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6460,7 +6460,7 @@
       <c r="M31" s="253"/>
       <c r="N31" s="135"/>
       <c r="O31" s="279"/>
-      <c r="P31" s="348"/>
+      <c r="P31" s="349"/>
       <c r="Q31" s="13"/>
     </row>
     <row r="32" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6499,7 +6499,7 @@
       <c r="M32" s="253"/>
       <c r="N32" s="135"/>
       <c r="O32" s="279"/>
-      <c r="P32" s="348"/>
+      <c r="P32" s="349"/>
       <c r="Q32" s="13"/>
     </row>
     <row r="33" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6538,7 +6538,7 @@
       <c r="M33" s="253"/>
       <c r="N33" s="135"/>
       <c r="O33" s="279"/>
-      <c r="P33" s="348"/>
+      <c r="P33" s="349"/>
       <c r="Q33" s="13"/>
     </row>
     <row r="34" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6577,7 +6577,7 @@
       <c r="M34" s="253"/>
       <c r="N34" s="135"/>
       <c r="O34" s="279"/>
-      <c r="P34" s="348"/>
+      <c r="P34" s="349"/>
       <c r="Q34" s="13"/>
     </row>
     <row r="35" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6616,7 +6616,7 @@
       <c r="M35" s="253"/>
       <c r="N35" s="135"/>
       <c r="O35" s="279"/>
-      <c r="P35" s="348"/>
+      <c r="P35" s="349"/>
       <c r="Q35" s="13"/>
     </row>
     <row r="36" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6655,7 +6655,7 @@
       <c r="M36" s="254"/>
       <c r="N36" s="146"/>
       <c r="O36" s="280"/>
-      <c r="P36" s="348"/>
+      <c r="P36" s="349"/>
       <c r="Q36" s="13"/>
     </row>
     <row r="37" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6694,7 +6694,7 @@
       <c r="M37" s="255"/>
       <c r="N37" s="155"/>
       <c r="O37" s="281"/>
-      <c r="P37" s="349" t="s">
+      <c r="P37" s="350" t="s">
         <v>13</v>
       </c>
       <c r="Q37" s="13"/>
@@ -6745,7 +6745,7 @@
       <c r="O38" s="282">
         <v>1</v>
       </c>
-      <c r="P38" s="349"/>
+      <c r="P38" s="350"/>
       <c r="Q38" s="13"/>
     </row>
     <row r="39" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6784,7 +6784,7 @@
       <c r="M39" s="256"/>
       <c r="N39" s="163"/>
       <c r="O39" s="282"/>
-      <c r="P39" s="349"/>
+      <c r="P39" s="350"/>
       <c r="Q39" s="13"/>
     </row>
     <row r="40" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6823,7 +6823,7 @@
       <c r="M40" s="256"/>
       <c r="N40" s="163"/>
       <c r="O40" s="282"/>
-      <c r="P40" s="349"/>
+      <c r="P40" s="350"/>
       <c r="Q40" s="13"/>
     </row>
     <row r="41" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6862,7 +6862,7 @@
       <c r="M41" s="257"/>
       <c r="N41" s="172"/>
       <c r="O41" s="283"/>
-      <c r="P41" s="349"/>
+      <c r="P41" s="350"/>
       <c r="Q41" s="13"/>
     </row>
     <row r="42" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -6911,7 +6911,7 @@
       <c r="O42" s="284">
         <v>1</v>
       </c>
-      <c r="P42" s="350" t="s">
+      <c r="P42" s="351" t="s">
         <v>34</v>
       </c>
       <c r="Q42" s="13"/>
@@ -6952,7 +6952,7 @@
       <c r="M43" s="259"/>
       <c r="N43" s="191"/>
       <c r="O43" s="285"/>
-      <c r="P43" s="351"/>
+      <c r="P43" s="352"/>
       <c r="Q43" s="13"/>
     </row>
     <row r="44" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -6991,7 +6991,7 @@
       <c r="M44" s="259"/>
       <c r="N44" s="191"/>
       <c r="O44" s="285"/>
-      <c r="P44" s="351"/>
+      <c r="P44" s="352"/>
       <c r="Q44" s="13"/>
     </row>
     <row r="45" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -7030,7 +7030,7 @@
       <c r="M45" s="259"/>
       <c r="N45" s="191"/>
       <c r="O45" s="285"/>
-      <c r="P45" s="351"/>
+      <c r="P45" s="352"/>
       <c r="Q45" s="13"/>
     </row>
     <row r="46" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -7079,7 +7079,7 @@
       <c r="O46" s="285">
         <v>1</v>
       </c>
-      <c r="P46" s="351"/>
+      <c r="P46" s="352"/>
       <c r="Q46" s="13"/>
     </row>
     <row r="47" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -7118,7 +7118,7 @@
       <c r="M47" s="259"/>
       <c r="N47" s="191"/>
       <c r="O47" s="285"/>
-      <c r="P47" s="351"/>
+      <c r="P47" s="352"/>
       <c r="Q47" s="13"/>
     </row>
     <row r="48" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -7157,7 +7157,7 @@
       <c r="M48" s="261"/>
       <c r="N48" s="199"/>
       <c r="O48" s="286"/>
-      <c r="P48" s="351"/>
+      <c r="P48" s="352"/>
       <c r="Q48" s="13"/>
     </row>
     <row r="49" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -7196,7 +7196,7 @@
       <c r="M49" s="262"/>
       <c r="N49" s="202"/>
       <c r="O49" s="287"/>
-      <c r="P49" s="352"/>
+      <c r="P49" s="353"/>
       <c r="Q49" s="13"/>
     </row>
     <row r="50" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -7234,7 +7234,7 @@
       <c r="M50" s="263"/>
       <c r="N50" s="211"/>
       <c r="O50" s="288"/>
-      <c r="P50" s="342" t="s">
+      <c r="P50" s="343" t="s">
         <v>28</v>
       </c>
       <c r="Q50" s="13"/>
@@ -7275,7 +7275,7 @@
       <c r="M51" s="264"/>
       <c r="N51" s="220"/>
       <c r="O51" s="289"/>
-      <c r="P51" s="342"/>
+      <c r="P51" s="343"/>
       <c r="Q51" s="13"/>
     </row>
     <row r="52" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -7314,7 +7314,7 @@
       <c r="M52" s="265"/>
       <c r="N52" s="230"/>
       <c r="O52" s="290"/>
-      <c r="P52" s="342"/>
+      <c r="P52" s="343"/>
       <c r="Q52" s="13"/>
     </row>
     <row r="53" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -7353,7 +7353,7 @@
       <c r="M53" s="265"/>
       <c r="N53" s="230"/>
       <c r="O53" s="290"/>
-      <c r="P53" s="342"/>
+      <c r="P53" s="343"/>
       <c r="Q53" s="13"/>
     </row>
     <row r="54" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -7392,7 +7392,7 @@
       <c r="M54" s="265"/>
       <c r="N54" s="230"/>
       <c r="O54" s="290"/>
-      <c r="P54" s="342"/>
+      <c r="P54" s="343"/>
       <c r="Q54" s="13"/>
     </row>
     <row r="55" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -7431,7 +7431,7 @@
       <c r="M55" s="265"/>
       <c r="N55" s="230"/>
       <c r="O55" s="290"/>
-      <c r="P55" s="342"/>
+      <c r="P55" s="343"/>
       <c r="Q55" s="13"/>
     </row>
     <row r="56" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -7470,7 +7470,7 @@
       <c r="M56" s="265"/>
       <c r="N56" s="230"/>
       <c r="O56" s="290"/>
-      <c r="P56" s="342"/>
+      <c r="P56" s="343"/>
       <c r="Q56" s="13"/>
     </row>
     <row r="57" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -7509,7 +7509,7 @@
       <c r="M57" s="265"/>
       <c r="N57" s="230"/>
       <c r="O57" s="290"/>
-      <c r="P57" s="342"/>
+      <c r="P57" s="343"/>
       <c r="Q57" s="13"/>
     </row>
     <row r="58" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -7548,7 +7548,7 @@
       <c r="M58" s="265"/>
       <c r="N58" s="230"/>
       <c r="O58" s="290"/>
-      <c r="P58" s="342"/>
+      <c r="P58" s="343"/>
       <c r="Q58" s="13"/>
     </row>
     <row r="59" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -7587,7 +7587,7 @@
       <c r="M59" s="265"/>
       <c r="N59" s="230"/>
       <c r="O59" s="290"/>
-      <c r="P59" s="342"/>
+      <c r="P59" s="343"/>
       <c r="Q59" s="13"/>
     </row>
     <row r="60" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -7626,7 +7626,7 @@
       <c r="M60" s="265"/>
       <c r="N60" s="230"/>
       <c r="O60" s="290"/>
-      <c r="P60" s="342"/>
+      <c r="P60" s="343"/>
       <c r="Q60" s="13"/>
     </row>
     <row r="61" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -7665,7 +7665,7 @@
       <c r="M61" s="266"/>
       <c r="N61" s="240"/>
       <c r="O61" s="291"/>
-      <c r="P61" s="342"/>
+      <c r="P61" s="343"/>
       <c r="Q61" s="13"/>
     </row>
     <row r="62" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -8125,7 +8125,7 @@
       <c r="M3" s="242"/>
       <c r="N3" s="43"/>
       <c r="O3" s="267"/>
-      <c r="P3" s="343" t="s">
+      <c r="P3" s="344" t="s">
         <v>31</v>
       </c>
       <c r="Q3" s="13"/>
@@ -8166,7 +8166,7 @@
       <c r="M4" s="243"/>
       <c r="N4" s="53"/>
       <c r="O4" s="268"/>
-      <c r="P4" s="343"/>
+      <c r="P4" s="344"/>
       <c r="Q4" s="13"/>
     </row>
     <row r="5" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8205,7 +8205,7 @@
       <c r="M5" s="244"/>
       <c r="N5" s="60"/>
       <c r="O5" s="269"/>
-      <c r="P5" s="343"/>
+      <c r="P5" s="344"/>
       <c r="Q5" s="13"/>
     </row>
     <row r="6" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8244,7 +8244,7 @@
       <c r="M6" s="244"/>
       <c r="N6" s="60"/>
       <c r="O6" s="269"/>
-      <c r="P6" s="343"/>
+      <c r="P6" s="344"/>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8283,7 +8283,7 @@
       <c r="M7" s="244"/>
       <c r="N7" s="60"/>
       <c r="O7" s="269"/>
-      <c r="P7" s="343"/>
+      <c r="P7" s="344"/>
       <c r="Q7" s="13"/>
     </row>
     <row r="8" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8322,7 +8322,7 @@
       <c r="M8" s="244"/>
       <c r="N8" s="60"/>
       <c r="O8" s="269"/>
-      <c r="P8" s="343"/>
+      <c r="P8" s="344"/>
       <c r="Q8" s="13"/>
     </row>
     <row r="9" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8361,7 +8361,7 @@
       <c r="M9" s="244"/>
       <c r="N9" s="60"/>
       <c r="O9" s="269"/>
-      <c r="P9" s="343"/>
+      <c r="P9" s="344"/>
       <c r="Q9" s="13"/>
     </row>
     <row r="10" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8400,7 +8400,7 @@
       <c r="M10" s="244"/>
       <c r="N10" s="60"/>
       <c r="O10" s="269"/>
-      <c r="P10" s="343"/>
+      <c r="P10" s="344"/>
       <c r="Q10" s="13"/>
     </row>
     <row r="11" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8449,7 +8449,7 @@
       <c r="O11" s="269">
         <v>2</v>
       </c>
-      <c r="P11" s="343"/>
+      <c r="P11" s="344"/>
       <c r="Q11" s="13"/>
     </row>
     <row r="12" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8488,7 +8488,7 @@
       <c r="M12" s="244"/>
       <c r="N12" s="60"/>
       <c r="O12" s="269"/>
-      <c r="P12" s="343"/>
+      <c r="P12" s="344"/>
       <c r="Q12" s="13"/>
     </row>
     <row r="13" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8537,7 +8537,7 @@
       <c r="O13" s="269">
         <v>2</v>
       </c>
-      <c r="P13" s="343"/>
+      <c r="P13" s="344"/>
       <c r="Q13" s="13"/>
     </row>
     <row r="14" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8586,7 +8586,7 @@
       <c r="O14" s="269">
         <v>1</v>
       </c>
-      <c r="P14" s="343"/>
+      <c r="P14" s="344"/>
       <c r="Q14" s="13"/>
     </row>
     <row r="15" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8625,7 +8625,7 @@
       <c r="M15" s="245"/>
       <c r="N15" s="67"/>
       <c r="O15" s="270"/>
-      <c r="P15" s="343"/>
+      <c r="P15" s="344"/>
       <c r="Q15" s="13"/>
     </row>
     <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -8674,7 +8674,7 @@
       <c r="O16" s="271">
         <v>4</v>
       </c>
-      <c r="P16" s="344" t="s">
+      <c r="P16" s="345" t="s">
         <v>12</v>
       </c>
       <c r="Q16" s="13"/>
@@ -8725,7 +8725,7 @@
       <c r="O17" s="272">
         <v>0</v>
       </c>
-      <c r="P17" s="345"/>
+      <c r="P17" s="346"/>
       <c r="Q17" s="13"/>
     </row>
     <row r="18" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -8774,7 +8774,7 @@
       <c r="O18" s="272">
         <v>11</v>
       </c>
-      <c r="P18" s="345"/>
+      <c r="P18" s="346"/>
       <c r="Q18" s="13"/>
     </row>
     <row r="19" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -8823,7 +8823,7 @@
       <c r="O19" s="272">
         <v>0</v>
       </c>
-      <c r="P19" s="345"/>
+      <c r="P19" s="346"/>
       <c r="Q19" s="13"/>
     </row>
     <row r="20" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -8862,7 +8862,7 @@
       <c r="M20" s="247"/>
       <c r="N20" s="83"/>
       <c r="O20" s="272"/>
-      <c r="P20" s="345"/>
+      <c r="P20" s="346"/>
       <c r="Q20" s="13"/>
     </row>
     <row r="21" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -8901,7 +8901,7 @@
       <c r="M21" s="247"/>
       <c r="N21" s="83"/>
       <c r="O21" s="272"/>
-      <c r="P21" s="345"/>
+      <c r="P21" s="346"/>
       <c r="Q21" s="13"/>
     </row>
     <row r="22" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -8940,7 +8940,7 @@
       <c r="M22" s="247"/>
       <c r="N22" s="83"/>
       <c r="O22" s="272"/>
-      <c r="P22" s="345"/>
+      <c r="P22" s="346"/>
       <c r="Q22" s="13"/>
     </row>
     <row r="23" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -8979,7 +8979,7 @@
       <c r="M23" s="247"/>
       <c r="N23" s="91"/>
       <c r="O23" s="273"/>
-      <c r="P23" s="345"/>
+      <c r="P23" s="346"/>
       <c r="Q23" s="13"/>
     </row>
     <row r="24" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9018,7 +9018,7 @@
       <c r="M24" s="248"/>
       <c r="N24" s="99"/>
       <c r="O24" s="274"/>
-      <c r="P24" s="346"/>
+      <c r="P24" s="347"/>
       <c r="Q24" s="13"/>
     </row>
     <row r="25" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9067,7 +9067,7 @@
       <c r="O25" s="275">
         <v>6</v>
       </c>
-      <c r="P25" s="347" t="s">
+      <c r="P25" s="348" t="s">
         <v>32</v>
       </c>
       <c r="Q25" s="13"/>
@@ -9118,7 +9118,7 @@
       <c r="O26" s="276">
         <v>9</v>
       </c>
-      <c r="P26" s="347"/>
+      <c r="P26" s="348"/>
       <c r="Q26" s="13"/>
     </row>
     <row r="27" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9167,7 +9167,7 @@
       <c r="O27" s="277">
         <v>1</v>
       </c>
-      <c r="P27" s="347"/>
+      <c r="P27" s="348"/>
       <c r="Q27" s="13"/>
     </row>
     <row r="28" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9216,7 +9216,7 @@
       <c r="O28" s="278">
         <v>24</v>
       </c>
-      <c r="P28" s="348" t="s">
+      <c r="P28" s="349" t="s">
         <v>33</v>
       </c>
       <c r="Q28" s="13"/>
@@ -9267,7 +9267,7 @@
       <c r="O29" s="279">
         <v>6</v>
       </c>
-      <c r="P29" s="348"/>
+      <c r="P29" s="349"/>
       <c r="Q29" s="13"/>
     </row>
     <row r="30" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9316,7 +9316,7 @@
       <c r="O30" s="279">
         <v>9</v>
       </c>
-      <c r="P30" s="348"/>
+      <c r="P30" s="349"/>
       <c r="Q30" s="13"/>
     </row>
     <row r="31" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9365,7 +9365,7 @@
       <c r="O31" s="279">
         <v>4</v>
       </c>
-      <c r="P31" s="348"/>
+      <c r="P31" s="349"/>
       <c r="Q31" s="13"/>
     </row>
     <row r="32" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9414,7 +9414,7 @@
       <c r="O32" s="279">
         <v>0</v>
       </c>
-      <c r="P32" s="348"/>
+      <c r="P32" s="349"/>
       <c r="Q32" s="13"/>
     </row>
     <row r="33" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9463,7 +9463,7 @@
       <c r="O33" s="279">
         <v>2</v>
       </c>
-      <c r="P33" s="348"/>
+      <c r="P33" s="349"/>
       <c r="Q33" s="13"/>
     </row>
     <row r="34" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9502,7 +9502,7 @@
       <c r="M34" s="253"/>
       <c r="N34" s="135"/>
       <c r="O34" s="279"/>
-      <c r="P34" s="348"/>
+      <c r="P34" s="349"/>
       <c r="Q34" s="13"/>
     </row>
     <row r="35" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9541,7 +9541,7 @@
       <c r="M35" s="253"/>
       <c r="N35" s="135"/>
       <c r="O35" s="279"/>
-      <c r="P35" s="348"/>
+      <c r="P35" s="349"/>
       <c r="Q35" s="13"/>
     </row>
     <row r="36" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9580,7 +9580,7 @@
       <c r="M36" s="254"/>
       <c r="N36" s="146"/>
       <c r="O36" s="280"/>
-      <c r="P36" s="348"/>
+      <c r="P36" s="349"/>
       <c r="Q36" s="13"/>
     </row>
     <row r="37" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9619,7 +9619,7 @@
       <c r="M37" s="255"/>
       <c r="N37" s="155"/>
       <c r="O37" s="281"/>
-      <c r="P37" s="349" t="s">
+      <c r="P37" s="350" t="s">
         <v>13</v>
       </c>
       <c r="Q37" s="13"/>
@@ -9670,7 +9670,7 @@
       <c r="O38" s="282">
         <v>0</v>
       </c>
-      <c r="P38" s="349"/>
+      <c r="P38" s="350"/>
       <c r="Q38" s="13"/>
     </row>
     <row r="39" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9719,7 +9719,7 @@
       <c r="O39" s="282">
         <v>3</v>
       </c>
-      <c r="P39" s="349"/>
+      <c r="P39" s="350"/>
       <c r="Q39" s="13"/>
     </row>
     <row r="40" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9768,7 +9768,7 @@
       <c r="O40" s="282">
         <v>1</v>
       </c>
-      <c r="P40" s="349"/>
+      <c r="P40" s="350"/>
       <c r="Q40" s="13"/>
     </row>
     <row r="41" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9817,7 +9817,7 @@
       <c r="O41" s="283">
         <v>3</v>
       </c>
-      <c r="P41" s="349"/>
+      <c r="P41" s="350"/>
       <c r="Q41" s="13"/>
     </row>
     <row r="42" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -9866,7 +9866,7 @@
       <c r="O42" s="284">
         <v>0</v>
       </c>
-      <c r="P42" s="350" t="s">
+      <c r="P42" s="351" t="s">
         <v>34</v>
       </c>
       <c r="Q42" s="13"/>
@@ -9917,7 +9917,7 @@
       <c r="O43" s="285">
         <v>2</v>
       </c>
-      <c r="P43" s="351"/>
+      <c r="P43" s="352"/>
       <c r="Q43" s="13"/>
     </row>
     <row r="44" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -9956,7 +9956,7 @@
       <c r="M44" s="259"/>
       <c r="N44" s="191"/>
       <c r="O44" s="285"/>
-      <c r="P44" s="351"/>
+      <c r="P44" s="352"/>
       <c r="Q44" s="13"/>
     </row>
     <row r="45" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -9995,7 +9995,7 @@
       <c r="M45" s="259"/>
       <c r="N45" s="191"/>
       <c r="O45" s="285"/>
-      <c r="P45" s="351"/>
+      <c r="P45" s="352"/>
       <c r="Q45" s="13"/>
     </row>
     <row r="46" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -10044,7 +10044,7 @@
       <c r="O46" s="285">
         <v>0</v>
       </c>
-      <c r="P46" s="351"/>
+      <c r="P46" s="352"/>
       <c r="Q46" s="13"/>
     </row>
     <row r="47" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -10083,7 +10083,7 @@
       <c r="M47" s="259"/>
       <c r="N47" s="191"/>
       <c r="O47" s="285"/>
-      <c r="P47" s="351"/>
+      <c r="P47" s="352"/>
       <c r="Q47" s="13"/>
     </row>
     <row r="48" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -10122,7 +10122,7 @@
       <c r="M48" s="261"/>
       <c r="N48" s="199"/>
       <c r="O48" s="286"/>
-      <c r="P48" s="351"/>
+      <c r="P48" s="352"/>
       <c r="Q48" s="13"/>
     </row>
     <row r="49" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -10161,7 +10161,7 @@
       <c r="M49" s="262"/>
       <c r="N49" s="202"/>
       <c r="O49" s="287"/>
-      <c r="P49" s="352"/>
+      <c r="P49" s="353"/>
       <c r="Q49" s="13"/>
     </row>
     <row r="50" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -10199,7 +10199,7 @@
       <c r="M50" s="263"/>
       <c r="N50" s="211"/>
       <c r="O50" s="288"/>
-      <c r="P50" s="342" t="s">
+      <c r="P50" s="343" t="s">
         <v>28</v>
       </c>
       <c r="Q50" s="13"/>
@@ -10240,7 +10240,7 @@
       <c r="M51" s="264"/>
       <c r="N51" s="220"/>
       <c r="O51" s="289"/>
-      <c r="P51" s="342"/>
+      <c r="P51" s="343"/>
       <c r="Q51" s="13"/>
     </row>
     <row r="52" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -10279,7 +10279,7 @@
       <c r="M52" s="265"/>
       <c r="N52" s="230"/>
       <c r="O52" s="290"/>
-      <c r="P52" s="342"/>
+      <c r="P52" s="343"/>
       <c r="Q52" s="13"/>
     </row>
     <row r="53" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -10318,7 +10318,7 @@
       <c r="M53" s="265"/>
       <c r="N53" s="230"/>
       <c r="O53" s="290"/>
-      <c r="P53" s="342"/>
+      <c r="P53" s="343"/>
       <c r="Q53" s="13"/>
     </row>
     <row r="54" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -10357,7 +10357,7 @@
       <c r="M54" s="265"/>
       <c r="N54" s="230"/>
       <c r="O54" s="290"/>
-      <c r="P54" s="342"/>
+      <c r="P54" s="343"/>
       <c r="Q54" s="13"/>
     </row>
     <row r="55" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -10396,7 +10396,7 @@
       <c r="M55" s="265"/>
       <c r="N55" s="230"/>
       <c r="O55" s="290"/>
-      <c r="P55" s="342"/>
+      <c r="P55" s="343"/>
       <c r="Q55" s="13"/>
     </row>
     <row r="56" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -10435,7 +10435,7 @@
       <c r="M56" s="265"/>
       <c r="N56" s="230"/>
       <c r="O56" s="290"/>
-      <c r="P56" s="342"/>
+      <c r="P56" s="343"/>
       <c r="Q56" s="13"/>
     </row>
     <row r="57" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -10474,7 +10474,7 @@
       <c r="M57" s="265"/>
       <c r="N57" s="230"/>
       <c r="O57" s="290"/>
-      <c r="P57" s="342"/>
+      <c r="P57" s="343"/>
       <c r="Q57" s="13"/>
     </row>
     <row r="58" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -10513,7 +10513,7 @@
       <c r="M58" s="265"/>
       <c r="N58" s="230"/>
       <c r="O58" s="290"/>
-      <c r="P58" s="342"/>
+      <c r="P58" s="343"/>
       <c r="Q58" s="13"/>
     </row>
     <row r="59" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -10552,7 +10552,7 @@
       <c r="M59" s="265"/>
       <c r="N59" s="230"/>
       <c r="O59" s="290"/>
-      <c r="P59" s="342"/>
+      <c r="P59" s="343"/>
       <c r="Q59" s="13"/>
     </row>
     <row r="60" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -10581,7 +10581,7 @@
       <c r="M60" s="299"/>
       <c r="N60" s="300"/>
       <c r="O60" s="301"/>
-      <c r="P60" s="342"/>
+      <c r="P60" s="343"/>
       <c r="Q60" s="13"/>
     </row>
     <row r="61" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -10620,7 +10620,7 @@
       <c r="M61" s="266"/>
       <c r="N61" s="240"/>
       <c r="O61" s="291"/>
-      <c r="P61" s="342"/>
+      <c r="P61" s="343"/>
       <c r="Q61" s="13"/>
     </row>
     <row r="62" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -11119,7 +11119,7 @@
       <c r="O3" s="267">
         <v>1</v>
       </c>
-      <c r="P3" s="343" t="s">
+      <c r="P3" s="344" t="s">
         <v>31</v>
       </c>
       <c r="Q3" s="13"/>
@@ -11160,7 +11160,7 @@
       <c r="M4" s="243"/>
       <c r="N4" s="53"/>
       <c r="O4" s="268"/>
-      <c r="P4" s="343"/>
+      <c r="P4" s="344"/>
       <c r="Q4" s="13"/>
     </row>
     <row r="5" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -11199,7 +11199,7 @@
       <c r="M5" s="244"/>
       <c r="N5" s="60"/>
       <c r="O5" s="269"/>
-      <c r="P5" s="343"/>
+      <c r="P5" s="344"/>
       <c r="Q5" s="13"/>
     </row>
     <row r="6" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -11238,7 +11238,7 @@
       <c r="M6" s="244"/>
       <c r="N6" s="60"/>
       <c r="O6" s="269"/>
-      <c r="P6" s="343"/>
+      <c r="P6" s="344"/>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -11277,7 +11277,7 @@
       <c r="M7" s="244"/>
       <c r="N7" s="60"/>
       <c r="O7" s="269"/>
-      <c r="P7" s="343"/>
+      <c r="P7" s="344"/>
       <c r="Q7" s="13"/>
     </row>
     <row r="8" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -11326,7 +11326,7 @@
       <c r="O8" s="269">
         <v>6</v>
       </c>
-      <c r="P8" s="343"/>
+      <c r="P8" s="344"/>
       <c r="Q8" s="13"/>
     </row>
     <row r="9" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -11365,7 +11365,7 @@
       <c r="M9" s="244"/>
       <c r="N9" s="60"/>
       <c r="O9" s="269"/>
-      <c r="P9" s="343"/>
+      <c r="P9" s="344"/>
       <c r="Q9" s="13"/>
     </row>
     <row r="10" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -11414,7 +11414,7 @@
       <c r="O10" s="269">
         <v>5</v>
       </c>
-      <c r="P10" s="343"/>
+      <c r="P10" s="344"/>
       <c r="Q10" s="13"/>
     </row>
     <row r="11" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -11463,7 +11463,7 @@
       <c r="O11" s="269">
         <v>0</v>
       </c>
-      <c r="P11" s="343"/>
+      <c r="P11" s="344"/>
       <c r="Q11" s="13"/>
     </row>
     <row r="12" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -11512,7 +11512,7 @@
       <c r="O12" s="269">
         <v>10</v>
       </c>
-      <c r="P12" s="343"/>
+      <c r="P12" s="344"/>
       <c r="Q12" s="13"/>
     </row>
     <row r="13" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -11561,7 +11561,7 @@
       <c r="O13" s="269">
         <v>2</v>
       </c>
-      <c r="P13" s="343"/>
+      <c r="P13" s="344"/>
       <c r="Q13" s="13"/>
     </row>
     <row r="14" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -11610,7 +11610,7 @@
       <c r="O14" s="269">
         <v>11</v>
       </c>
-      <c r="P14" s="343"/>
+      <c r="P14" s="344"/>
       <c r="Q14" s="13"/>
     </row>
     <row r="15" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -11659,7 +11659,7 @@
       <c r="O15" s="270">
         <v>6</v>
       </c>
-      <c r="P15" s="343"/>
+      <c r="P15" s="344"/>
       <c r="Q15" s="13"/>
     </row>
     <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -11708,7 +11708,7 @@
       <c r="O16" s="271">
         <v>14</v>
       </c>
-      <c r="P16" s="344" t="s">
+      <c r="P16" s="345" t="s">
         <v>12</v>
       </c>
       <c r="Q16" s="13"/>
@@ -11739,7 +11739,7 @@
       <c r="M17" s="299"/>
       <c r="N17" s="300"/>
       <c r="O17" s="301"/>
-      <c r="P17" s="345"/>
+      <c r="P17" s="346"/>
       <c r="Q17" s="13"/>
     </row>
     <row r="18" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -11768,7 +11768,7 @@
       <c r="M18" s="299"/>
       <c r="N18" s="300"/>
       <c r="O18" s="301"/>
-      <c r="P18" s="345"/>
+      <c r="P18" s="346"/>
       <c r="Q18" s="13"/>
     </row>
     <row r="19" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -11797,7 +11797,7 @@
       <c r="M19" s="299"/>
       <c r="N19" s="300"/>
       <c r="O19" s="301"/>
-      <c r="P19" s="345"/>
+      <c r="P19" s="346"/>
       <c r="Q19" s="13"/>
     </row>
     <row r="20" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -11826,7 +11826,7 @@
       <c r="M20" s="299"/>
       <c r="N20" s="300"/>
       <c r="O20" s="301"/>
-      <c r="P20" s="345"/>
+      <c r="P20" s="346"/>
       <c r="Q20" s="13"/>
     </row>
     <row r="21" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -11855,7 +11855,7 @@
       <c r="M21" s="299"/>
       <c r="N21" s="300"/>
       <c r="O21" s="301"/>
-      <c r="P21" s="345"/>
+      <c r="P21" s="346"/>
       <c r="Q21" s="13"/>
     </row>
     <row r="22" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -11884,7 +11884,7 @@
       <c r="M22" s="299"/>
       <c r="N22" s="300"/>
       <c r="O22" s="301"/>
-      <c r="P22" s="345"/>
+      <c r="P22" s="346"/>
       <c r="Q22" s="13"/>
     </row>
     <row r="23" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -11913,7 +11913,7 @@
       <c r="M23" s="299"/>
       <c r="N23" s="307"/>
       <c r="O23" s="308"/>
-      <c r="P23" s="345"/>
+      <c r="P23" s="346"/>
       <c r="Q23" s="13"/>
     </row>
     <row r="24" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -11942,7 +11942,7 @@
       <c r="M24" s="314"/>
       <c r="N24" s="315"/>
       <c r="O24" s="316"/>
-      <c r="P24" s="346"/>
+      <c r="P24" s="347"/>
       <c r="Q24" s="13"/>
     </row>
     <row r="25" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -11991,7 +11991,7 @@
       <c r="O25" s="275">
         <v>47</v>
       </c>
-      <c r="P25" s="347" t="s">
+      <c r="P25" s="348" t="s">
         <v>32</v>
       </c>
       <c r="Q25" s="13"/>
@@ -12042,7 +12042,7 @@
       <c r="O26" s="276">
         <v>6</v>
       </c>
-      <c r="P26" s="347"/>
+      <c r="P26" s="348"/>
       <c r="Q26" s="13"/>
     </row>
     <row r="27" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -12091,7 +12091,7 @@
       <c r="O27" s="277">
         <v>116</v>
       </c>
-      <c r="P27" s="347"/>
+      <c r="P27" s="348"/>
       <c r="Q27" s="13"/>
     </row>
     <row r="28" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -12140,7 +12140,7 @@
       <c r="O28" s="278">
         <v>17</v>
       </c>
-      <c r="P28" s="348" t="s">
+      <c r="P28" s="349" t="s">
         <v>33</v>
       </c>
       <c r="Q28" s="13"/>
@@ -12191,7 +12191,7 @@
       <c r="O29" s="279">
         <v>41</v>
       </c>
-      <c r="P29" s="348"/>
+      <c r="P29" s="349"/>
       <c r="Q29" s="13"/>
     </row>
     <row r="30" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -12240,7 +12240,7 @@
       <c r="O30" s="279">
         <v>1</v>
       </c>
-      <c r="P30" s="348"/>
+      <c r="P30" s="349"/>
       <c r="Q30" s="13"/>
     </row>
     <row r="31" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -12289,7 +12289,7 @@
       <c r="O31" s="279">
         <v>6</v>
       </c>
-      <c r="P31" s="348"/>
+      <c r="P31" s="349"/>
       <c r="Q31" s="13"/>
     </row>
     <row r="32" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -12338,7 +12338,7 @@
       <c r="O32" s="279">
         <v>4</v>
       </c>
-      <c r="P32" s="348"/>
+      <c r="P32" s="349"/>
       <c r="Q32" s="13"/>
     </row>
     <row r="33" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -12387,7 +12387,7 @@
       <c r="O33" s="279">
         <v>0</v>
       </c>
-      <c r="P33" s="348"/>
+      <c r="P33" s="349"/>
       <c r="Q33" s="13"/>
     </row>
     <row r="34" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -12436,7 +12436,7 @@
       <c r="O34" s="279">
         <v>1</v>
       </c>
-      <c r="P34" s="348"/>
+      <c r="P34" s="349"/>
       <c r="Q34" s="13"/>
     </row>
     <row r="35" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -12475,7 +12475,7 @@
       <c r="M35" s="253"/>
       <c r="N35" s="135"/>
       <c r="O35" s="279"/>
-      <c r="P35" s="348"/>
+      <c r="P35" s="349"/>
       <c r="Q35" s="13"/>
     </row>
     <row r="36" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -12524,7 +12524,7 @@
       <c r="O36" s="280">
         <v>0</v>
       </c>
-      <c r="P36" s="348"/>
+      <c r="P36" s="349"/>
       <c r="Q36" s="13"/>
     </row>
     <row r="37" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -12573,7 +12573,7 @@
       <c r="O37" s="281">
         <v>4</v>
       </c>
-      <c r="P37" s="349" t="s">
+      <c r="P37" s="350" t="s">
         <v>13</v>
       </c>
       <c r="Q37" s="13"/>
@@ -12624,7 +12624,7 @@
       <c r="O38" s="282">
         <v>1</v>
       </c>
-      <c r="P38" s="349"/>
+      <c r="P38" s="350"/>
       <c r="Q38" s="13"/>
     </row>
     <row r="39" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -12673,7 +12673,7 @@
       <c r="O39" s="282">
         <v>2</v>
       </c>
-      <c r="P39" s="349"/>
+      <c r="P39" s="350"/>
       <c r="Q39" s="13"/>
     </row>
     <row r="40" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -12722,7 +12722,7 @@
       <c r="O40" s="282">
         <v>2</v>
       </c>
-      <c r="P40" s="349"/>
+      <c r="P40" s="350"/>
       <c r="Q40" s="13"/>
     </row>
     <row r="41" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -12771,7 +12771,7 @@
       <c r="O41" s="283">
         <v>2</v>
       </c>
-      <c r="P41" s="349"/>
+      <c r="P41" s="350"/>
       <c r="Q41" s="13"/>
     </row>
     <row r="42" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -12810,7 +12810,7 @@
       <c r="M42" s="258"/>
       <c r="N42" s="182"/>
       <c r="O42" s="284"/>
-      <c r="P42" s="350" t="s">
+      <c r="P42" s="351" t="s">
         <v>34</v>
       </c>
       <c r="Q42" s="13"/>
@@ -12851,7 +12851,7 @@
       <c r="M43" s="259"/>
       <c r="N43" s="191"/>
       <c r="O43" s="285"/>
-      <c r="P43" s="351"/>
+      <c r="P43" s="352"/>
       <c r="Q43" s="13"/>
     </row>
     <row r="44" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -12890,7 +12890,7 @@
       <c r="M44" s="259"/>
       <c r="N44" s="191"/>
       <c r="O44" s="285"/>
-      <c r="P44" s="351"/>
+      <c r="P44" s="352"/>
       <c r="Q44" s="13"/>
     </row>
     <row r="45" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -12929,7 +12929,7 @@
       <c r="M45" s="259"/>
       <c r="N45" s="191"/>
       <c r="O45" s="285"/>
-      <c r="P45" s="351"/>
+      <c r="P45" s="352"/>
       <c r="Q45" s="13"/>
     </row>
     <row r="46" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -12968,7 +12968,7 @@
       <c r="M46" s="259"/>
       <c r="N46" s="191"/>
       <c r="O46" s="285"/>
-      <c r="P46" s="351"/>
+      <c r="P46" s="352"/>
       <c r="Q46" s="13"/>
     </row>
     <row r="47" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -13007,7 +13007,7 @@
       <c r="M47" s="259"/>
       <c r="N47" s="191"/>
       <c r="O47" s="285"/>
-      <c r="P47" s="351"/>
+      <c r="P47" s="352"/>
       <c r="Q47" s="13"/>
     </row>
     <row r="48" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -13046,7 +13046,7 @@
       <c r="M48" s="261"/>
       <c r="N48" s="199"/>
       <c r="O48" s="286"/>
-      <c r="P48" s="351"/>
+      <c r="P48" s="352"/>
       <c r="Q48" s="13"/>
     </row>
     <row r="49" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -13085,7 +13085,7 @@
       <c r="M49" s="262"/>
       <c r="N49" s="202"/>
       <c r="O49" s="287"/>
-      <c r="P49" s="352"/>
+      <c r="P49" s="353"/>
       <c r="Q49" s="13"/>
     </row>
     <row r="50" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -13133,7 +13133,7 @@
       <c r="O50" s="288">
         <v>0</v>
       </c>
-      <c r="P50" s="342" t="s">
+      <c r="P50" s="343" t="s">
         <v>28</v>
       </c>
       <c r="Q50" s="13"/>
@@ -13174,7 +13174,7 @@
       <c r="M51" s="264"/>
       <c r="N51" s="220"/>
       <c r="O51" s="289"/>
-      <c r="P51" s="342"/>
+      <c r="P51" s="343"/>
       <c r="Q51" s="13"/>
     </row>
     <row r="52" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -13213,7 +13213,7 @@
       <c r="M52" s="265"/>
       <c r="N52" s="230"/>
       <c r="O52" s="290"/>
-      <c r="P52" s="342"/>
+      <c r="P52" s="343"/>
       <c r="Q52" s="13"/>
     </row>
     <row r="53" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -13252,7 +13252,7 @@
       <c r="M53" s="265"/>
       <c r="N53" s="230"/>
       <c r="O53" s="290"/>
-      <c r="P53" s="342"/>
+      <c r="P53" s="343"/>
       <c r="Q53" s="13"/>
     </row>
     <row r="54" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -13291,7 +13291,7 @@
       <c r="M54" s="265"/>
       <c r="N54" s="230"/>
       <c r="O54" s="290"/>
-      <c r="P54" s="342"/>
+      <c r="P54" s="343"/>
       <c r="Q54" s="13"/>
     </row>
     <row r="55" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -13330,7 +13330,7 @@
       <c r="M55" s="265"/>
       <c r="N55" s="230"/>
       <c r="O55" s="290"/>
-      <c r="P55" s="342"/>
+      <c r="P55" s="343"/>
       <c r="Q55" s="13"/>
     </row>
     <row r="56" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -13369,7 +13369,7 @@
       <c r="M56" s="265"/>
       <c r="N56" s="230"/>
       <c r="O56" s="290"/>
-      <c r="P56" s="342"/>
+      <c r="P56" s="343"/>
       <c r="Q56" s="13"/>
     </row>
     <row r="57" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -13408,7 +13408,7 @@
       <c r="M57" s="265"/>
       <c r="N57" s="230"/>
       <c r="O57" s="290"/>
-      <c r="P57" s="342"/>
+      <c r="P57" s="343"/>
       <c r="Q57" s="13"/>
     </row>
     <row r="58" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -13447,7 +13447,7 @@
       <c r="M58" s="265"/>
       <c r="N58" s="230"/>
       <c r="O58" s="290"/>
-      <c r="P58" s="342"/>
+      <c r="P58" s="343"/>
       <c r="Q58" s="13"/>
     </row>
     <row r="59" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -13486,7 +13486,7 @@
       <c r="M59" s="265"/>
       <c r="N59" s="230"/>
       <c r="O59" s="290"/>
-      <c r="P59" s="342"/>
+      <c r="P59" s="343"/>
       <c r="Q59" s="13"/>
     </row>
     <row r="60" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -13525,7 +13525,7 @@
       <c r="M60" s="265"/>
       <c r="N60" s="230"/>
       <c r="O60" s="290"/>
-      <c r="P60" s="342"/>
+      <c r="P60" s="343"/>
       <c r="Q60" s="13"/>
     </row>
     <row r="61" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -13564,7 +13564,7 @@
       <c r="M61" s="266"/>
       <c r="N61" s="240"/>
       <c r="O61" s="291"/>
-      <c r="P61" s="342"/>
+      <c r="P61" s="343"/>
       <c r="Q61" s="13"/>
     </row>
     <row r="62" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -14065,7 +14065,7 @@
       <c r="M3" s="242"/>
       <c r="N3" s="43"/>
       <c r="O3" s="267"/>
-      <c r="P3" s="343" t="s">
+      <c r="P3" s="344" t="s">
         <v>31</v>
       </c>
       <c r="Q3" s="13"/>
@@ -14104,7 +14104,7 @@
       <c r="M4" s="243"/>
       <c r="N4" s="53"/>
       <c r="O4" s="268"/>
-      <c r="P4" s="343"/>
+      <c r="P4" s="344"/>
       <c r="Q4" s="13"/>
     </row>
     <row r="5" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -14141,7 +14141,7 @@
       <c r="M5" s="244"/>
       <c r="N5" s="60"/>
       <c r="O5" s="269"/>
-      <c r="P5" s="343"/>
+      <c r="P5" s="344"/>
       <c r="Q5" s="13"/>
     </row>
     <row r="6" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -14178,7 +14178,7 @@
       <c r="M6" s="244"/>
       <c r="N6" s="60"/>
       <c r="O6" s="269"/>
-      <c r="P6" s="343"/>
+      <c r="P6" s="344"/>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -14215,7 +14215,7 @@
       <c r="M7" s="244"/>
       <c r="N7" s="60"/>
       <c r="O7" s="269"/>
-      <c r="P7" s="343"/>
+      <c r="P7" s="344"/>
       <c r="Q7" s="13"/>
     </row>
     <row r="8" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -14260,7 +14260,7 @@
       <c r="O8" s="269">
         <v>2</v>
       </c>
-      <c r="P8" s="343"/>
+      <c r="P8" s="344"/>
       <c r="Q8" s="13"/>
     </row>
     <row r="9" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -14305,7 +14305,7 @@
         <v>30.6666666666667</v>
       </c>
       <c r="O9" s="269"/>
-      <c r="P9" s="343"/>
+      <c r="P9" s="344"/>
       <c r="Q9" s="13"/>
     </row>
     <row r="10" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -14352,7 +14352,7 @@
       <c r="O10" s="269">
         <v>5</v>
       </c>
-      <c r="P10" s="343"/>
+      <c r="P10" s="344"/>
       <c r="Q10" s="13"/>
     </row>
     <row r="11" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -14399,7 +14399,7 @@
       <c r="O11" s="269">
         <v>4</v>
       </c>
-      <c r="P11" s="343"/>
+      <c r="P11" s="344"/>
       <c r="Q11" s="13"/>
     </row>
     <row r="12" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -14446,7 +14446,7 @@
       <c r="O12" s="269">
         <v>0</v>
       </c>
-      <c r="P12" s="343"/>
+      <c r="P12" s="344"/>
       <c r="Q12" s="13"/>
     </row>
     <row r="13" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -14493,7 +14493,7 @@
       <c r="O13" s="269">
         <v>4</v>
       </c>
-      <c r="P13" s="343"/>
+      <c r="P13" s="344"/>
       <c r="Q13" s="13"/>
     </row>
     <row r="14" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -14538,7 +14538,7 @@
       <c r="O14" s="269">
         <v>11</v>
       </c>
-      <c r="P14" s="343"/>
+      <c r="P14" s="344"/>
       <c r="Q14" s="13"/>
     </row>
     <row r="15" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -14583,7 +14583,7 @@
       <c r="O15" s="270">
         <v>15</v>
       </c>
-      <c r="P15" s="343"/>
+      <c r="P15" s="344"/>
       <c r="Q15" s="13"/>
     </row>
     <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -14628,7 +14628,7 @@
       <c r="O16" s="271">
         <v>8</v>
       </c>
-      <c r="P16" s="344" t="s">
+      <c r="P16" s="345" t="s">
         <v>12</v>
       </c>
       <c r="Q16" s="13"/>
@@ -14677,7 +14677,7 @@
       <c r="O17" s="272">
         <v>16</v>
       </c>
-      <c r="P17" s="345"/>
+      <c r="P17" s="346"/>
       <c r="Q17" s="13"/>
     </row>
     <row r="18" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -14724,7 +14724,7 @@
       <c r="O18" s="272">
         <v>22</v>
       </c>
-      <c r="P18" s="345"/>
+      <c r="P18" s="346"/>
       <c r="Q18" s="13"/>
     </row>
     <row r="19" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -14771,7 +14771,7 @@
       <c r="O19" s="272">
         <v>43</v>
       </c>
-      <c r="P19" s="345"/>
+      <c r="P19" s="346"/>
       <c r="Q19" s="13"/>
     </row>
     <row r="20" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -14818,7 +14818,7 @@
       <c r="O20" s="272">
         <v>20</v>
       </c>
-      <c r="P20" s="345"/>
+      <c r="P20" s="346"/>
       <c r="Q20" s="13"/>
     </row>
     <row r="21" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -14865,7 +14865,7 @@
       <c r="O21" s="272">
         <v>14</v>
       </c>
-      <c r="P21" s="345"/>
+      <c r="P21" s="346"/>
       <c r="Q21" s="13"/>
     </row>
     <row r="22" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -14912,7 +14912,7 @@
       <c r="O22" s="272">
         <v>51</v>
       </c>
-      <c r="P22" s="345"/>
+      <c r="P22" s="346"/>
       <c r="Q22" s="13"/>
     </row>
     <row r="23" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -14959,7 +14959,7 @@
       <c r="O23" s="273">
         <v>15</v>
       </c>
-      <c r="P23" s="345"/>
+      <c r="P23" s="346"/>
       <c r="Q23" s="13"/>
     </row>
     <row r="24" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15006,7 +15006,7 @@
       <c r="O24" s="274">
         <v>0</v>
       </c>
-      <c r="P24" s="346"/>
+      <c r="P24" s="347"/>
       <c r="Q24" s="13"/>
     </row>
     <row r="25" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15051,7 +15051,7 @@
       <c r="O25" s="275">
         <v>21</v>
       </c>
-      <c r="P25" s="347" t="s">
+      <c r="P25" s="348" t="s">
         <v>32</v>
       </c>
       <c r="Q25" s="13"/>
@@ -15100,7 +15100,7 @@
       <c r="O26" s="276">
         <v>22</v>
       </c>
-      <c r="P26" s="347"/>
+      <c r="P26" s="348"/>
       <c r="Q26" s="13"/>
     </row>
     <row r="27" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15147,7 +15147,7 @@
       <c r="O27" s="277">
         <v>12</v>
       </c>
-      <c r="P27" s="347"/>
+      <c r="P27" s="348"/>
       <c r="Q27" s="13"/>
     </row>
     <row r="28" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15192,7 +15192,7 @@
       <c r="O28" s="278">
         <v>33</v>
       </c>
-      <c r="P28" s="348" t="s">
+      <c r="P28" s="349" t="s">
         <v>33</v>
       </c>
       <c r="Q28" s="13"/>
@@ -15239,7 +15239,7 @@
       <c r="O29" s="279">
         <v>17</v>
       </c>
-      <c r="P29" s="348"/>
+      <c r="P29" s="349"/>
       <c r="Q29" s="13"/>
     </row>
     <row r="30" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15286,7 +15286,7 @@
       <c r="O30" s="279">
         <v>49</v>
       </c>
-      <c r="P30" s="348"/>
+      <c r="P30" s="349"/>
       <c r="Q30" s="13"/>
     </row>
     <row r="31" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15331,7 +15331,7 @@
       <c r="O31" s="279">
         <v>26</v>
       </c>
-      <c r="P31" s="348"/>
+      <c r="P31" s="349"/>
       <c r="Q31" s="13"/>
     </row>
     <row r="32" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15378,7 +15378,7 @@
       <c r="O32" s="279">
         <v>13</v>
       </c>
-      <c r="P32" s="348"/>
+      <c r="P32" s="349"/>
       <c r="Q32" s="13"/>
     </row>
     <row r="33" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15425,7 +15425,7 @@
       <c r="O33" s="279">
         <v>39</v>
       </c>
-      <c r="P33" s="348"/>
+      <c r="P33" s="349"/>
       <c r="Q33" s="13"/>
     </row>
     <row r="34" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15472,7 +15472,7 @@
       <c r="O34" s="279">
         <v>76</v>
       </c>
-      <c r="P34" s="348"/>
+      <c r="P34" s="349"/>
       <c r="Q34" s="13"/>
     </row>
     <row r="35" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15519,7 +15519,7 @@
       <c r="O35" s="279">
         <v>2</v>
       </c>
-      <c r="P35" s="348"/>
+      <c r="P35" s="349"/>
       <c r="Q35" s="13"/>
     </row>
     <row r="36" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15566,7 +15566,7 @@
       <c r="O36" s="280">
         <v>3</v>
       </c>
-      <c r="P36" s="348"/>
+      <c r="P36" s="349"/>
       <c r="Q36" s="13"/>
     </row>
     <row r="37" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15613,7 +15613,7 @@
       <c r="O37" s="281">
         <v>33</v>
       </c>
-      <c r="P37" s="349" t="s">
+      <c r="P37" s="350" t="s">
         <v>13</v>
       </c>
       <c r="Q37" s="13"/>
@@ -15662,7 +15662,7 @@
       <c r="O38" s="282">
         <v>26</v>
       </c>
-      <c r="P38" s="349"/>
+      <c r="P38" s="350"/>
       <c r="Q38" s="13"/>
     </row>
     <row r="39" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15709,7 +15709,7 @@
       <c r="O39" s="282">
         <v>6</v>
       </c>
-      <c r="P39" s="349"/>
+      <c r="P39" s="350"/>
       <c r="Q39" s="13"/>
     </row>
     <row r="40" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15754,7 +15754,7 @@
       <c r="O40" s="282">
         <v>4</v>
       </c>
-      <c r="P40" s="349"/>
+      <c r="P40" s="350"/>
       <c r="Q40" s="13"/>
     </row>
     <row r="41" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -15801,7 +15801,7 @@
       <c r="O41" s="283">
         <v>9</v>
       </c>
-      <c r="P41" s="349"/>
+      <c r="P41" s="350"/>
       <c r="Q41" s="13"/>
     </row>
     <row r="42" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -15848,7 +15848,7 @@
       <c r="O42" s="284">
         <v>0</v>
       </c>
-      <c r="P42" s="350" t="s">
+      <c r="P42" s="351" t="s">
         <v>34</v>
       </c>
       <c r="Q42" s="13"/>
@@ -15897,7 +15897,7 @@
       <c r="O43" s="285">
         <v>8</v>
       </c>
-      <c r="P43" s="351"/>
+      <c r="P43" s="352"/>
       <c r="Q43" s="13"/>
     </row>
     <row r="44" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -15944,7 +15944,7 @@
       <c r="O44" s="285">
         <v>4</v>
       </c>
-      <c r="P44" s="351"/>
+      <c r="P44" s="352"/>
       <c r="Q44" s="13"/>
     </row>
     <row r="45" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -15991,7 +15991,7 @@
       <c r="O45" s="285">
         <v>1</v>
       </c>
-      <c r="P45" s="351"/>
+      <c r="P45" s="352"/>
       <c r="Q45" s="13"/>
     </row>
     <row r="46" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -16038,7 +16038,7 @@
       <c r="O46" s="285">
         <v>3</v>
       </c>
-      <c r="P46" s="351"/>
+      <c r="P46" s="352"/>
       <c r="Q46" s="13"/>
     </row>
     <row r="47" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -16075,7 +16075,7 @@
       <c r="M47" s="259"/>
       <c r="N47" s="191"/>
       <c r="O47" s="285"/>
-      <c r="P47" s="351"/>
+      <c r="P47" s="352"/>
       <c r="Q47" s="13"/>
     </row>
     <row r="48" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -16112,7 +16112,7 @@
       <c r="M48" s="261"/>
       <c r="N48" s="199"/>
       <c r="O48" s="286"/>
-      <c r="P48" s="351"/>
+      <c r="P48" s="352"/>
       <c r="Q48" s="13"/>
     </row>
     <row r="49" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -16159,7 +16159,7 @@
       <c r="O49" s="287">
         <v>2</v>
       </c>
-      <c r="P49" s="352"/>
+      <c r="P49" s="353"/>
       <c r="Q49" s="13"/>
     </row>
     <row r="50" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -16206,7 +16206,7 @@
       <c r="O50" s="288">
         <v>0</v>
       </c>
-      <c r="P50" s="342" t="s">
+      <c r="P50" s="343" t="s">
         <v>28</v>
       </c>
       <c r="Q50" s="13"/>
@@ -16255,7 +16255,7 @@
       <c r="O51" s="289">
         <v>2</v>
       </c>
-      <c r="P51" s="342"/>
+      <c r="P51" s="343"/>
       <c r="Q51" s="13"/>
     </row>
     <row r="52" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -16302,7 +16302,7 @@
       <c r="O52" s="290">
         <v>2</v>
       </c>
-      <c r="P52" s="342"/>
+      <c r="P52" s="343"/>
       <c r="Q52" s="13"/>
     </row>
     <row r="53" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -16349,7 +16349,7 @@
       <c r="O53" s="290">
         <v>2</v>
       </c>
-      <c r="P53" s="342"/>
+      <c r="P53" s="343"/>
       <c r="Q53" s="13"/>
     </row>
     <row r="54" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -16386,7 +16386,7 @@
       <c r="M54" s="265"/>
       <c r="N54" s="230"/>
       <c r="O54" s="290"/>
-      <c r="P54" s="342"/>
+      <c r="P54" s="343"/>
       <c r="Q54" s="13"/>
     </row>
     <row r="55" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -16423,7 +16423,7 @@
       <c r="M55" s="265"/>
       <c r="N55" s="230"/>
       <c r="O55" s="290"/>
-      <c r="P55" s="342"/>
+      <c r="P55" s="343"/>
       <c r="Q55" s="13"/>
     </row>
     <row r="56" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -16460,7 +16460,7 @@
       <c r="M56" s="265"/>
       <c r="N56" s="230"/>
       <c r="O56" s="290"/>
-      <c r="P56" s="342"/>
+      <c r="P56" s="343"/>
       <c r="Q56" s="13"/>
     </row>
     <row r="57" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -16497,7 +16497,7 @@
       <c r="M57" s="265"/>
       <c r="N57" s="230"/>
       <c r="O57" s="290"/>
-      <c r="P57" s="342"/>
+      <c r="P57" s="343"/>
       <c r="Q57" s="13"/>
     </row>
     <row r="58" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -16534,7 +16534,7 @@
       <c r="M58" s="265"/>
       <c r="N58" s="230"/>
       <c r="O58" s="290"/>
-      <c r="P58" s="342"/>
+      <c r="P58" s="343"/>
       <c r="Q58" s="13"/>
     </row>
     <row r="59" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -16571,7 +16571,7 @@
       <c r="M59" s="265"/>
       <c r="N59" s="230"/>
       <c r="O59" s="290"/>
-      <c r="P59" s="342"/>
+      <c r="P59" s="343"/>
       <c r="Q59" s="13"/>
     </row>
     <row r="60" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -16608,7 +16608,7 @@
       <c r="M60" s="265"/>
       <c r="N60" s="230"/>
       <c r="O60" s="290"/>
-      <c r="P60" s="342"/>
+      <c r="P60" s="343"/>
       <c r="Q60" s="13"/>
     </row>
     <row r="61" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -16645,7 +16645,7 @@
       <c r="M61" s="266"/>
       <c r="N61" s="240"/>
       <c r="O61" s="291"/>
-      <c r="P61" s="342"/>
+      <c r="P61" s="343"/>
       <c r="Q61" s="13"/>
     </row>
     <row r="62" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -17141,7 +17141,7 @@
       <c r="M3" s="242"/>
       <c r="N3" s="43"/>
       <c r="O3" s="267"/>
-      <c r="P3" s="343" t="s">
+      <c r="P3" s="344" t="s">
         <v>31</v>
       </c>
       <c r="Q3" s="13"/>
@@ -17182,7 +17182,7 @@
       <c r="M4" s="243"/>
       <c r="N4" s="53"/>
       <c r="O4" s="268"/>
-      <c r="P4" s="343"/>
+      <c r="P4" s="344"/>
       <c r="Q4" s="13"/>
     </row>
     <row r="5" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -17221,7 +17221,7 @@
       <c r="M5" s="244"/>
       <c r="N5" s="60"/>
       <c r="O5" s="269"/>
-      <c r="P5" s="343"/>
+      <c r="P5" s="344"/>
       <c r="Q5" s="13"/>
     </row>
     <row r="6" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -17260,7 +17260,7 @@
       <c r="M6" s="244"/>
       <c r="N6" s="60"/>
       <c r="O6" s="269"/>
-      <c r="P6" s="343"/>
+      <c r="P6" s="344"/>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -17299,7 +17299,7 @@
       <c r="M7" s="244"/>
       <c r="N7" s="60"/>
       <c r="O7" s="269"/>
-      <c r="P7" s="343"/>
+      <c r="P7" s="344"/>
       <c r="Q7" s="13"/>
     </row>
     <row r="8" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -17348,7 +17348,7 @@
       <c r="O8" s="269">
         <v>5</v>
       </c>
-      <c r="P8" s="343"/>
+      <c r="P8" s="344"/>
       <c r="Q8" s="13"/>
     </row>
     <row r="9" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -17387,7 +17387,7 @@
       <c r="M9" s="244"/>
       <c r="N9" s="60"/>
       <c r="O9" s="269"/>
-      <c r="P9" s="343"/>
+      <c r="P9" s="344"/>
       <c r="Q9" s="13"/>
     </row>
     <row r="10" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -17436,7 +17436,7 @@
       <c r="O10" s="269">
         <v>2</v>
       </c>
-      <c r="P10" s="343"/>
+      <c r="P10" s="344"/>
       <c r="Q10" s="13"/>
     </row>
     <row r="11" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -17485,7 +17485,7 @@
       <c r="O11" s="269">
         <v>0</v>
       </c>
-      <c r="P11" s="343"/>
+      <c r="P11" s="344"/>
       <c r="Q11" s="13"/>
     </row>
     <row r="12" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -17524,7 +17524,7 @@
       <c r="M12" s="244"/>
       <c r="N12" s="60"/>
       <c r="O12" s="269"/>
-      <c r="P12" s="343"/>
+      <c r="P12" s="344"/>
       <c r="Q12" s="13"/>
     </row>
     <row r="13" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -17573,7 +17573,7 @@
       <c r="O13" s="269">
         <v>2</v>
       </c>
-      <c r="P13" s="343"/>
+      <c r="P13" s="344"/>
       <c r="Q13" s="13"/>
     </row>
     <row r="14" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -17612,7 +17612,7 @@
       <c r="M14" s="244"/>
       <c r="N14" s="60"/>
       <c r="O14" s="269"/>
-      <c r="P14" s="343"/>
+      <c r="P14" s="344"/>
       <c r="Q14" s="13"/>
     </row>
     <row r="15" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -17651,7 +17651,7 @@
       <c r="M15" s="245"/>
       <c r="N15" s="67"/>
       <c r="O15" s="270"/>
-      <c r="P15" s="343"/>
+      <c r="P15" s="344"/>
       <c r="Q15" s="13"/>
     </row>
     <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -17700,7 +17700,7 @@
       <c r="O16" s="271">
         <v>50</v>
       </c>
-      <c r="P16" s="344" t="s">
+      <c r="P16" s="345" t="s">
         <v>12</v>
       </c>
       <c r="Q16" s="13"/>
@@ -17751,7 +17751,7 @@
       <c r="O17" s="272">
         <v>0</v>
       </c>
-      <c r="P17" s="345"/>
+      <c r="P17" s="346"/>
       <c r="Q17" s="13"/>
     </row>
     <row r="18" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -17800,7 +17800,7 @@
       <c r="O18" s="272">
         <v>1</v>
       </c>
-      <c r="P18" s="345"/>
+      <c r="P18" s="346"/>
       <c r="Q18" s="13"/>
     </row>
     <row r="19" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -17849,7 +17849,7 @@
       <c r="O19" s="272">
         <v>6</v>
       </c>
-      <c r="P19" s="345"/>
+      <c r="P19" s="346"/>
       <c r="Q19" s="13"/>
     </row>
     <row r="20" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -17898,7 +17898,7 @@
       <c r="O20" s="272">
         <v>1</v>
       </c>
-      <c r="P20" s="345"/>
+      <c r="P20" s="346"/>
       <c r="Q20" s="13"/>
     </row>
     <row r="21" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -17947,7 +17947,7 @@
       <c r="O21" s="272">
         <v>41</v>
       </c>
-      <c r="P21" s="345"/>
+      <c r="P21" s="346"/>
       <c r="Q21" s="13"/>
     </row>
     <row r="22" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -17996,7 +17996,7 @@
       <c r="O22" s="272">
         <v>5</v>
       </c>
-      <c r="P22" s="345"/>
+      <c r="P22" s="346"/>
       <c r="Q22" s="13"/>
     </row>
     <row r="23" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -18045,7 +18045,7 @@
       <c r="O23" s="273">
         <v>0</v>
       </c>
-      <c r="P23" s="345"/>
+      <c r="P23" s="346"/>
       <c r="Q23" s="13"/>
     </row>
     <row r="24" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18094,7 +18094,7 @@
       <c r="O24" s="274">
         <v>12</v>
       </c>
-      <c r="P24" s="346"/>
+      <c r="P24" s="347"/>
       <c r="Q24" s="13"/>
     </row>
     <row r="25" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18133,7 +18133,7 @@
       <c r="M25" s="249"/>
       <c r="N25" s="107"/>
       <c r="O25" s="275"/>
-      <c r="P25" s="347" t="s">
+      <c r="P25" s="348" t="s">
         <v>32</v>
       </c>
       <c r="Q25" s="13"/>
@@ -18184,7 +18184,7 @@
       <c r="O26" s="276">
         <v>1</v>
       </c>
-      <c r="P26" s="347"/>
+      <c r="P26" s="348"/>
       <c r="Q26" s="13"/>
     </row>
     <row r="27" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18223,7 +18223,7 @@
       <c r="M27" s="251"/>
       <c r="N27" s="121"/>
       <c r="O27" s="277"/>
-      <c r="P27" s="347"/>
+      <c r="P27" s="348"/>
       <c r="Q27" s="13"/>
     </row>
     <row r="28" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18270,7 +18270,7 @@
       <c r="O28" s="278">
         <v>536</v>
       </c>
-      <c r="P28" s="348" t="s">
+      <c r="P28" s="349" t="s">
         <v>33</v>
       </c>
       <c r="Q28" s="13"/>
@@ -18321,7 +18321,7 @@
       <c r="O29" s="279">
         <v>55</v>
       </c>
-      <c r="P29" s="348"/>
+      <c r="P29" s="349"/>
       <c r="Q29" s="13"/>
     </row>
     <row r="30" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18370,7 +18370,7 @@
       <c r="O30" s="279">
         <v>168</v>
       </c>
-      <c r="P30" s="348"/>
+      <c r="P30" s="349"/>
       <c r="Q30" s="13"/>
     </row>
     <row r="31" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18419,7 +18419,7 @@
       <c r="O31" s="279">
         <v>28</v>
       </c>
-      <c r="P31" s="348"/>
+      <c r="P31" s="349"/>
       <c r="Q31" s="13"/>
     </row>
     <row r="32" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18468,7 +18468,7 @@
       <c r="O32" s="279">
         <v>44</v>
       </c>
-      <c r="P32" s="348"/>
+      <c r="P32" s="349"/>
       <c r="Q32" s="13"/>
     </row>
     <row r="33" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18517,7 +18517,7 @@
       <c r="O33" s="279">
         <v>23</v>
       </c>
-      <c r="P33" s="348"/>
+      <c r="P33" s="349"/>
       <c r="Q33" s="13"/>
     </row>
     <row r="34" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18566,7 +18566,7 @@
       <c r="O34" s="279">
         <v>52</v>
       </c>
-      <c r="P34" s="348"/>
+      <c r="P34" s="349"/>
       <c r="Q34" s="13"/>
     </row>
     <row r="35" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18615,7 +18615,7 @@
       <c r="O35" s="279">
         <v>10</v>
       </c>
-      <c r="P35" s="348"/>
+      <c r="P35" s="349"/>
       <c r="Q35" s="13"/>
     </row>
     <row r="36" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18664,7 +18664,7 @@
       <c r="O36" s="280">
         <v>10</v>
       </c>
-      <c r="P36" s="348"/>
+      <c r="P36" s="349"/>
       <c r="Q36" s="13"/>
     </row>
     <row r="37" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18713,7 +18713,7 @@
       <c r="O37" s="281">
         <v>161</v>
       </c>
-      <c r="P37" s="349" t="s">
+      <c r="P37" s="350" t="s">
         <v>13</v>
       </c>
       <c r="Q37" s="13"/>
@@ -18764,7 +18764,7 @@
       <c r="O38" s="282">
         <v>27</v>
       </c>
-      <c r="P38" s="349"/>
+      <c r="P38" s="350"/>
       <c r="Q38" s="13"/>
     </row>
     <row r="39" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18813,7 +18813,7 @@
       <c r="O39" s="282">
         <v>19</v>
       </c>
-      <c r="P39" s="349"/>
+      <c r="P39" s="350"/>
       <c r="Q39" s="13"/>
     </row>
     <row r="40" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18862,7 +18862,7 @@
       <c r="O40" s="282">
         <v>0</v>
       </c>
-      <c r="P40" s="349"/>
+      <c r="P40" s="350"/>
       <c r="Q40" s="13"/>
     </row>
     <row r="41" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18911,7 +18911,7 @@
       <c r="O41" s="283">
         <v>0</v>
       </c>
-      <c r="P41" s="349"/>
+      <c r="P41" s="350"/>
       <c r="Q41" s="13"/>
     </row>
     <row r="42" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -18960,7 +18960,7 @@
       <c r="O42" s="284">
         <v>0</v>
       </c>
-      <c r="P42" s="350" t="s">
+      <c r="P42" s="351" t="s">
         <v>34</v>
       </c>
       <c r="Q42" s="13"/>
@@ -19011,7 +19011,7 @@
       <c r="O43" s="285">
         <v>9</v>
       </c>
-      <c r="P43" s="351"/>
+      <c r="P43" s="352"/>
       <c r="Q43" s="13"/>
     </row>
     <row r="44" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -19060,7 +19060,7 @@
       <c r="O44" s="285">
         <v>0</v>
       </c>
-      <c r="P44" s="351"/>
+      <c r="P44" s="352"/>
       <c r="Q44" s="13"/>
     </row>
     <row r="45" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -19109,7 +19109,7 @@
       <c r="O45" s="285">
         <v>9</v>
       </c>
-      <c r="P45" s="351"/>
+      <c r="P45" s="352"/>
       <c r="Q45" s="13"/>
     </row>
     <row r="46" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -19158,7 +19158,7 @@
       <c r="O46" s="285">
         <v>6</v>
       </c>
-      <c r="P46" s="351"/>
+      <c r="P46" s="352"/>
       <c r="Q46" s="13"/>
     </row>
     <row r="47" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -19197,7 +19197,7 @@
       <c r="M47" s="259"/>
       <c r="N47" s="191"/>
       <c r="O47" s="285"/>
-      <c r="P47" s="351"/>
+      <c r="P47" s="352"/>
       <c r="Q47" s="13"/>
     </row>
     <row r="48" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -19246,7 +19246,7 @@
       <c r="O48" s="286">
         <v>1</v>
       </c>
-      <c r="P48" s="351"/>
+      <c r="P48" s="352"/>
       <c r="Q48" s="13"/>
     </row>
     <row r="49" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -19295,7 +19295,7 @@
       <c r="O49" s="287">
         <v>1</v>
       </c>
-      <c r="P49" s="352"/>
+      <c r="P49" s="353"/>
       <c r="Q49" s="13"/>
     </row>
     <row r="50" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -19343,7 +19343,7 @@
       <c r="O50" s="288">
         <v>11</v>
       </c>
-      <c r="P50" s="342" t="s">
+      <c r="P50" s="343" t="s">
         <v>28</v>
       </c>
       <c r="Q50" s="13"/>
@@ -19394,7 +19394,7 @@
       <c r="O51" s="289">
         <v>4</v>
       </c>
-      <c r="P51" s="342"/>
+      <c r="P51" s="343"/>
       <c r="Q51" s="13"/>
     </row>
     <row r="52" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -19443,7 +19443,7 @@
       <c r="O52" s="290">
         <v>0</v>
       </c>
-      <c r="P52" s="342"/>
+      <c r="P52" s="343"/>
       <c r="Q52" s="13"/>
     </row>
     <row r="53" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -19492,7 +19492,7 @@
       <c r="O53" s="290">
         <v>0</v>
       </c>
-      <c r="P53" s="342"/>
+      <c r="P53" s="343"/>
       <c r="Q53" s="13"/>
     </row>
     <row r="54" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -19531,7 +19531,7 @@
       <c r="M54" s="265"/>
       <c r="N54" s="230"/>
       <c r="O54" s="290"/>
-      <c r="P54" s="342"/>
+      <c r="P54" s="343"/>
       <c r="Q54" s="13"/>
     </row>
     <row r="55" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -19570,7 +19570,7 @@
       <c r="M55" s="265"/>
       <c r="N55" s="230"/>
       <c r="O55" s="290"/>
-      <c r="P55" s="342"/>
+      <c r="P55" s="343"/>
       <c r="Q55" s="13"/>
     </row>
     <row r="56" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -19609,7 +19609,7 @@
       <c r="M56" s="265"/>
       <c r="N56" s="230"/>
       <c r="O56" s="290"/>
-      <c r="P56" s="342"/>
+      <c r="P56" s="343"/>
       <c r="Q56" s="13"/>
     </row>
     <row r="57" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -19648,7 +19648,7 @@
       <c r="M57" s="265"/>
       <c r="N57" s="230"/>
       <c r="O57" s="290"/>
-      <c r="P57" s="342"/>
+      <c r="P57" s="343"/>
       <c r="Q57" s="13"/>
     </row>
     <row r="58" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -19697,7 +19697,7 @@
       <c r="O58" s="290">
         <v>0</v>
       </c>
-      <c r="P58" s="342"/>
+      <c r="P58" s="343"/>
       <c r="Q58" s="13"/>
     </row>
     <row r="59" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -19736,7 +19736,7 @@
       <c r="M59" s="265"/>
       <c r="N59" s="230"/>
       <c r="O59" s="290"/>
-      <c r="P59" s="342"/>
+      <c r="P59" s="343"/>
       <c r="Q59" s="13"/>
     </row>
     <row r="60" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -19775,7 +19775,7 @@
       <c r="M60" s="265"/>
       <c r="N60" s="230"/>
       <c r="O60" s="290"/>
-      <c r="P60" s="342"/>
+      <c r="P60" s="343"/>
       <c r="Q60" s="13"/>
     </row>
     <row r="61" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -19814,7 +19814,7 @@
       <c r="M61" s="266"/>
       <c r="N61" s="240"/>
       <c r="O61" s="291"/>
-      <c r="P61" s="342"/>
+      <c r="P61" s="343"/>
       <c r="Q61" s="13"/>
     </row>
     <row r="62" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -19825,7 +19825,7 @@
       <c r="C62" s="5"/>
       <c r="D62" s="5"/>
       <c r="E62" s="5"/>
-      <c r="F62" s="354"/>
+      <c r="F62" s="342"/>
       <c r="G62"/>
       <c r="H62"/>
       <c r="I62"/>
@@ -20268,7 +20268,7 @@
       <c r="M3" s="242"/>
       <c r="N3" s="43"/>
       <c r="O3" s="267"/>
-      <c r="P3" s="343" t="s">
+      <c r="P3" s="344" t="s">
         <v>31</v>
       </c>
       <c r="Q3" s="13"/>
@@ -20297,7 +20297,7 @@
       <c r="M4" s="243"/>
       <c r="N4" s="53"/>
       <c r="O4" s="268"/>
-      <c r="P4" s="343"/>
+      <c r="P4" s="344"/>
       <c r="Q4" s="13"/>
     </row>
     <row r="5" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -20324,7 +20324,7 @@
       <c r="M5" s="244"/>
       <c r="N5" s="60"/>
       <c r="O5" s="269"/>
-      <c r="P5" s="343"/>
+      <c r="P5" s="344"/>
       <c r="Q5" s="13"/>
     </row>
     <row r="6" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -20373,7 +20373,7 @@
       <c r="O6" s="269">
         <v>8</v>
       </c>
-      <c r="P6" s="343"/>
+      <c r="P6" s="344"/>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -20400,7 +20400,7 @@
       <c r="M7" s="244"/>
       <c r="N7" s="60"/>
       <c r="O7" s="269"/>
-      <c r="P7" s="343"/>
+      <c r="P7" s="344"/>
       <c r="Q7" s="13"/>
     </row>
     <row r="8" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -20427,7 +20427,7 @@
       <c r="M8" s="244"/>
       <c r="N8" s="60"/>
       <c r="O8" s="269"/>
-      <c r="P8" s="343"/>
+      <c r="P8" s="344"/>
       <c r="Q8" s="13"/>
     </row>
     <row r="9" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -20454,7 +20454,7 @@
       <c r="M9" s="244"/>
       <c r="N9" s="60"/>
       <c r="O9" s="269"/>
-      <c r="P9" s="343"/>
+      <c r="P9" s="344"/>
       <c r="Q9" s="13"/>
     </row>
     <row r="10" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -20481,7 +20481,7 @@
       <c r="M10" s="244"/>
       <c r="N10" s="60"/>
       <c r="O10" s="269"/>
-      <c r="P10" s="343"/>
+      <c r="P10" s="344"/>
       <c r="Q10" s="13"/>
     </row>
     <row r="11" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -20508,7 +20508,7 @@
       <c r="M11" s="244"/>
       <c r="N11" s="60"/>
       <c r="O11" s="269"/>
-      <c r="P11" s="343"/>
+      <c r="P11" s="344"/>
       <c r="Q11" s="13"/>
     </row>
     <row r="12" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -20535,7 +20535,7 @@
       <c r="M12" s="244"/>
       <c r="N12" s="60"/>
       <c r="O12" s="269"/>
-      <c r="P12" s="343"/>
+      <c r="P12" s="344"/>
       <c r="Q12" s="13"/>
     </row>
     <row r="13" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -20562,7 +20562,7 @@
       <c r="M13" s="244"/>
       <c r="N13" s="60"/>
       <c r="O13" s="269"/>
-      <c r="P13" s="343"/>
+      <c r="P13" s="344"/>
       <c r="Q13" s="13"/>
     </row>
     <row r="14" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -20589,7 +20589,7 @@
       <c r="M14" s="244"/>
       <c r="N14" s="60"/>
       <c r="O14" s="269"/>
-      <c r="P14" s="343"/>
+      <c r="P14" s="344"/>
       <c r="Q14" s="13"/>
     </row>
     <row r="15" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -20616,7 +20616,7 @@
       <c r="M15" s="245"/>
       <c r="N15" s="67"/>
       <c r="O15" s="270"/>
-      <c r="P15" s="343"/>
+      <c r="P15" s="344"/>
       <c r="Q15" s="13"/>
     </row>
     <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -20665,7 +20665,7 @@
       <c r="O16" s="271">
         <v>43</v>
       </c>
-      <c r="P16" s="344" t="s">
+      <c r="P16" s="345" t="s">
         <v>12</v>
       </c>
       <c r="Q16" s="13"/>
@@ -20694,7 +20694,7 @@
       <c r="M17" s="247"/>
       <c r="N17" s="83"/>
       <c r="O17" s="272"/>
-      <c r="P17" s="345"/>
+      <c r="P17" s="346"/>
       <c r="Q17" s="13"/>
     </row>
     <row r="18" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -20741,7 +20741,7 @@
       <c r="O18" s="272">
         <v>47</v>
       </c>
-      <c r="P18" s="345"/>
+      <c r="P18" s="346"/>
       <c r="Q18" s="13"/>
     </row>
     <row r="19" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -20788,7 +20788,7 @@
       <c r="O19" s="272">
         <v>14</v>
       </c>
-      <c r="P19" s="345"/>
+      <c r="P19" s="346"/>
       <c r="Q19" s="13"/>
     </row>
     <row r="20" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -20815,7 +20815,7 @@
       <c r="M20" s="247"/>
       <c r="N20" s="83"/>
       <c r="O20" s="272"/>
-      <c r="P20" s="345"/>
+      <c r="P20" s="346"/>
       <c r="Q20" s="13"/>
     </row>
     <row r="21" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -20842,7 +20842,7 @@
       <c r="M21" s="247"/>
       <c r="N21" s="83"/>
       <c r="O21" s="272"/>
-      <c r="P21" s="345"/>
+      <c r="P21" s="346"/>
       <c r="Q21" s="13"/>
     </row>
     <row r="22" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -20883,7 +20883,7 @@
       <c r="M22" s="247"/>
       <c r="N22" s="83"/>
       <c r="O22" s="272"/>
-      <c r="P22" s="345"/>
+      <c r="P22" s="346"/>
       <c r="Q22" s="13"/>
     </row>
     <row r="23" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -20910,7 +20910,7 @@
       <c r="M23" s="247"/>
       <c r="N23" s="91"/>
       <c r="O23" s="273"/>
-      <c r="P23" s="345"/>
+      <c r="P23" s="346"/>
       <c r="Q23" s="13"/>
     </row>
     <row r="24" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -20949,7 +20949,7 @@
       <c r="M24" s="248"/>
       <c r="N24" s="99"/>
       <c r="O24" s="274"/>
-      <c r="P24" s="346"/>
+      <c r="P24" s="347"/>
       <c r="Q24" s="13"/>
     </row>
     <row r="25" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -20976,7 +20976,7 @@
       <c r="M25" s="249"/>
       <c r="N25" s="107"/>
       <c r="O25" s="275"/>
-      <c r="P25" s="347" t="s">
+      <c r="P25" s="348" t="s">
         <v>32</v>
       </c>
       <c r="Q25" s="13"/>
@@ -21025,7 +21025,7 @@
       <c r="O26" s="276">
         <v>64</v>
       </c>
-      <c r="P26" s="347"/>
+      <c r="P26" s="348"/>
       <c r="Q26" s="13"/>
     </row>
     <row r="27" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -21074,7 +21074,7 @@
       <c r="O27" s="277">
         <v>8</v>
       </c>
-      <c r="P27" s="347"/>
+      <c r="P27" s="348"/>
       <c r="Q27" s="13"/>
     </row>
     <row r="28" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -21101,7 +21101,7 @@
       <c r="M28" s="252"/>
       <c r="N28" s="128"/>
       <c r="O28" s="278"/>
-      <c r="P28" s="348" t="s">
+      <c r="P28" s="349" t="s">
         <v>33</v>
       </c>
       <c r="Q28" s="13"/>
@@ -21152,7 +21152,7 @@
       <c r="O29" s="279">
         <v>37</v>
       </c>
-      <c r="P29" s="348"/>
+      <c r="P29" s="349"/>
       <c r="Q29" s="13"/>
     </row>
     <row r="30" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -21201,7 +21201,7 @@
       <c r="O30" s="279">
         <v>23</v>
       </c>
-      <c r="P30" s="348"/>
+      <c r="P30" s="349"/>
       <c r="Q30" s="13"/>
     </row>
     <row r="31" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -21228,7 +21228,7 @@
       <c r="M31" s="253"/>
       <c r="N31" s="135"/>
       <c r="O31" s="279"/>
-      <c r="P31" s="348"/>
+      <c r="P31" s="349"/>
       <c r="Q31" s="13"/>
     </row>
     <row r="32" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -21277,7 +21277,7 @@
       <c r="O32" s="279">
         <v>23</v>
       </c>
-      <c r="P32" s="348"/>
+      <c r="P32" s="349"/>
       <c r="Q32" s="13"/>
     </row>
     <row r="33" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -21326,7 +21326,7 @@
       <c r="O33" s="279">
         <v>10</v>
       </c>
-      <c r="P33" s="348"/>
+      <c r="P33" s="349"/>
       <c r="Q33" s="13"/>
     </row>
     <row r="34" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -21375,7 +21375,7 @@
       <c r="O34" s="279">
         <v>0</v>
       </c>
-      <c r="P34" s="348"/>
+      <c r="P34" s="349"/>
       <c r="Q34" s="13"/>
     </row>
     <row r="35" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -21414,7 +21414,7 @@
       <c r="M35" s="253"/>
       <c r="N35" s="135"/>
       <c r="O35" s="279"/>
-      <c r="P35" s="348"/>
+      <c r="P35" s="349"/>
       <c r="Q35" s="13"/>
     </row>
     <row r="36" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -21453,7 +21453,7 @@
       <c r="M36" s="254"/>
       <c r="N36" s="146"/>
       <c r="O36" s="280"/>
-      <c r="P36" s="348"/>
+      <c r="P36" s="349"/>
       <c r="Q36" s="13"/>
     </row>
     <row r="37" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -21502,7 +21502,7 @@
       <c r="O37" s="281">
         <v>11</v>
       </c>
-      <c r="P37" s="349" t="s">
+      <c r="P37" s="350" t="s">
         <v>13</v>
       </c>
       <c r="Q37" s="13"/>
@@ -21553,7 +21553,7 @@
       <c r="O38" s="282">
         <v>19</v>
       </c>
-      <c r="P38" s="349"/>
+      <c r="P38" s="350"/>
       <c r="Q38" s="13"/>
     </row>
     <row r="39" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -21602,7 +21602,7 @@
       <c r="O39" s="282">
         <v>10</v>
       </c>
-      <c r="P39" s="349"/>
+      <c r="P39" s="350"/>
       <c r="Q39" s="13"/>
     </row>
     <row r="40" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -21651,7 +21651,7 @@
       <c r="O40" s="282">
         <v>3</v>
       </c>
-      <c r="P40" s="349"/>
+      <c r="P40" s="350"/>
       <c r="Q40" s="13"/>
     </row>
     <row r="41" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -21690,7 +21690,7 @@
       <c r="M41" s="257"/>
       <c r="N41" s="172"/>
       <c r="O41" s="283"/>
-      <c r="P41" s="349"/>
+      <c r="P41" s="350"/>
       <c r="Q41" s="13"/>
     </row>
     <row r="42" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -21739,7 +21739,7 @@
       <c r="O42" s="284">
         <v>3</v>
       </c>
-      <c r="P42" s="350" t="s">
+      <c r="P42" s="351" t="s">
         <v>34</v>
       </c>
       <c r="Q42" s="13"/>
@@ -21790,7 +21790,7 @@
       <c r="O43" s="285">
         <v>8</v>
       </c>
-      <c r="P43" s="351"/>
+      <c r="P43" s="352"/>
       <c r="Q43" s="13"/>
     </row>
     <row r="44" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -21839,7 +21839,7 @@
       <c r="O44" s="285">
         <v>3</v>
       </c>
-      <c r="P44" s="351"/>
+      <c r="P44" s="352"/>
       <c r="Q44" s="13"/>
     </row>
     <row r="45" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -21888,7 +21888,7 @@
       <c r="O45" s="285">
         <v>3</v>
       </c>
-      <c r="P45" s="351"/>
+      <c r="P45" s="352"/>
       <c r="Q45" s="13"/>
     </row>
     <row r="46" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -21937,7 +21937,7 @@
       <c r="O46" s="285">
         <v>1</v>
       </c>
-      <c r="P46" s="351"/>
+      <c r="P46" s="352"/>
       <c r="Q46" s="13"/>
     </row>
     <row r="47" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -21976,7 +21976,7 @@
       <c r="M47" s="259"/>
       <c r="N47" s="191"/>
       <c r="O47" s="285"/>
-      <c r="P47" s="351"/>
+      <c r="P47" s="352"/>
       <c r="Q47" s="13"/>
     </row>
     <row r="48" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -22025,7 +22025,7 @@
       <c r="O48" s="286">
         <v>2</v>
       </c>
-      <c r="P48" s="351"/>
+      <c r="P48" s="352"/>
       <c r="Q48" s="13"/>
     </row>
     <row r="49" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -22064,7 +22064,7 @@
       <c r="M49" s="262"/>
       <c r="N49" s="202"/>
       <c r="O49" s="287"/>
-      <c r="P49" s="352"/>
+      <c r="P49" s="353"/>
       <c r="Q49" s="13"/>
     </row>
     <row r="50" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -22112,7 +22112,7 @@
       <c r="O50" s="288">
         <v>2</v>
       </c>
-      <c r="P50" s="342" t="s">
+      <c r="P50" s="343" t="s">
         <v>28</v>
       </c>
       <c r="Q50" s="13"/>
@@ -22153,7 +22153,7 @@
       <c r="M51" s="264"/>
       <c r="N51" s="220"/>
       <c r="O51" s="289"/>
-      <c r="P51" s="342"/>
+      <c r="P51" s="343"/>
       <c r="Q51" s="13"/>
     </row>
     <row r="52" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -22192,7 +22192,7 @@
       <c r="M52" s="265"/>
       <c r="N52" s="230"/>
       <c r="O52" s="290"/>
-      <c r="P52" s="342"/>
+      <c r="P52" s="343"/>
       <c r="Q52" s="13"/>
     </row>
     <row r="53" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -22231,7 +22231,7 @@
       <c r="M53" s="265"/>
       <c r="N53" s="230"/>
       <c r="O53" s="290"/>
-      <c r="P53" s="342"/>
+      <c r="P53" s="343"/>
       <c r="Q53" s="13"/>
     </row>
     <row r="54" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -22270,7 +22270,7 @@
       <c r="M54" s="265"/>
       <c r="N54" s="230"/>
       <c r="O54" s="290"/>
-      <c r="P54" s="342"/>
+      <c r="P54" s="343"/>
       <c r="Q54" s="13"/>
     </row>
     <row r="55" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -22309,7 +22309,7 @@
       <c r="M55" s="265"/>
       <c r="N55" s="230"/>
       <c r="O55" s="290"/>
-      <c r="P55" s="342"/>
+      <c r="P55" s="343"/>
       <c r="Q55" s="13"/>
     </row>
     <row r="56" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -22348,7 +22348,7 @@
       <c r="M56" s="265"/>
       <c r="N56" s="230"/>
       <c r="O56" s="290"/>
-      <c r="P56" s="342"/>
+      <c r="P56" s="343"/>
       <c r="Q56" s="13"/>
     </row>
     <row r="57" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -22387,7 +22387,7 @@
       <c r="M57" s="265"/>
       <c r="N57" s="230"/>
       <c r="O57" s="290"/>
-      <c r="P57" s="342"/>
+      <c r="P57" s="343"/>
       <c r="Q57" s="13"/>
     </row>
     <row r="58" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -22426,7 +22426,7 @@
       <c r="M58" s="265"/>
       <c r="N58" s="230"/>
       <c r="O58" s="290"/>
-      <c r="P58" s="342"/>
+      <c r="P58" s="343"/>
       <c r="Q58" s="13"/>
     </row>
     <row r="59" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -22465,7 +22465,7 @@
       <c r="M59" s="265"/>
       <c r="N59" s="230"/>
       <c r="O59" s="290"/>
-      <c r="P59" s="342"/>
+      <c r="P59" s="343"/>
       <c r="Q59" s="13"/>
     </row>
     <row r="60" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -22504,7 +22504,7 @@
       <c r="M60" s="265"/>
       <c r="N60" s="230"/>
       <c r="O60" s="290"/>
-      <c r="P60" s="342"/>
+      <c r="P60" s="343"/>
       <c r="Q60" s="13"/>
     </row>
     <row r="61" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -22543,7 +22543,7 @@
       <c r="M61" s="266"/>
       <c r="N61" s="240"/>
       <c r="O61" s="291"/>
-      <c r="P61" s="342"/>
+      <c r="P61" s="343"/>
       <c r="Q61" s="13"/>
     </row>
     <row r="62" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -22554,7 +22554,7 @@
       <c r="C62" s="5"/>
       <c r="D62" s="5"/>
       <c r="E62" s="5"/>
-      <c r="F62" s="1"/>
+      <c r="F62" s="342"/>
       <c r="G62"/>
       <c r="H62"/>
       <c r="I62"/>
@@ -22880,19 +22880,19 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:14" ht="24.6" x14ac:dyDescent="0.4">
-      <c r="A1" s="353" t="s">
+      <c r="A1" s="354" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="353"/>
-      <c r="C1" s="353"/>
-      <c r="D1" s="353"/>
-      <c r="E1" s="353"/>
-      <c r="F1" s="353"/>
-      <c r="G1" s="353"/>
-      <c r="H1" s="353"/>
-      <c r="I1" s="353"/>
-      <c r="J1" s="353"/>
-      <c r="K1" s="353"/>
+      <c r="B1" s="354"/>
+      <c r="C1" s="354"/>
+      <c r="D1" s="354"/>
+      <c r="E1" s="354"/>
+      <c r="F1" s="354"/>
+      <c r="G1" s="354"/>
+      <c r="H1" s="354"/>
+      <c r="I1" s="354"/>
+      <c r="J1" s="354"/>
+      <c r="K1" s="354"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="N2" s="339"/>

</xml_diff>